<commit_message>
Update IGCSE chemistry question bank
</commit_message>
<xml_diff>
--- a/data/question-bank.xlsx
+++ b/data/question-bank.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adamsun/Documents/Codex/2026-08-19/referenced-chatgpt-conversation-this-is-an/outputs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adamsun/Documents/Codex/2026-08-19/referenced-chatgpt-conversation-this-is-an/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B22365E-24DA-644B-9BFB-FF4F659B7573}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{890B0292-0C67-B44B-A489-F56554744CF9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1320" yWindow="600" windowWidth="28200" windowHeight="15100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="600" yWindow="600" windowWidth="28200" windowHeight="15100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Question Bank" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1027" uniqueCount="665">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1103" uniqueCount="726">
   <si>
     <t>id</t>
   </si>
@@ -1384,9 +1384,6 @@
     <t>Same functional group</t>
   </si>
   <si>
-    <t>Differ from one member to the next by -CH2-</t>
-  </si>
-  <si>
     <t>Similar chemical properties</t>
   </si>
   <si>
@@ -1475,9 +1472,6 @@
   </si>
   <si>
     <t>High temperature</t>
-  </si>
-  <si>
-    <t>Al2O3 catalyst</t>
   </si>
   <si>
     <t>CIE135</t>
@@ -2029,6 +2023,241 @@
   </si>
   <si>
     <t>4 Improvements</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Al₂O₃ catalyst</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Differ from one member to the next by -CH₂-</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>CIE184</t>
+  </si>
+  <si>
+    <t>CIE185</t>
+  </si>
+  <si>
+    <t>CIE186</t>
+  </si>
+  <si>
+    <t>CIE187</t>
+  </si>
+  <si>
+    <t>CIE188</t>
+  </si>
+  <si>
+    <t>CIE189</t>
+  </si>
+  <si>
+    <t>CIE190</t>
+  </si>
+  <si>
+    <t>CIE191</t>
+  </si>
+  <si>
+    <t>CIE192</t>
+  </si>
+  <si>
+    <t>CIE193</t>
+  </si>
+  <si>
+    <t>CIE194</t>
+  </si>
+  <si>
+    <t>CIE195</t>
+  </si>
+  <si>
+    <t>CIE196</t>
+  </si>
+  <si>
+    <t>CIE197</t>
+  </si>
+  <si>
+    <t>5 Lab apparatus</t>
+  </si>
+  <si>
+    <t>5 Lab apparatus</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Translate: conical flask</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Translate: measuring cylinder</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Translate: volumetric pipette</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Translate: burette</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Translate: beaker</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Translate: test tube</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Translate: boiling tube</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Translate: water bath</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Translate: glass rod</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Translate: condenser</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Translate: funnel</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Translate: gas syringe</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Translate: pestle and mortar</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Translate: Bunsen burner</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>CIE198</t>
+  </si>
+  <si>
+    <t>CIE199</t>
+  </si>
+  <si>
+    <t>Translate: crucible</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Translate: delivery tube</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>锥形瓶</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>量筒</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>容量移液管</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>滴定管</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>烧杯</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>试管</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>沸腾试管</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>水浴盆</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>玻璃棒</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>冷凝器</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>漏斗</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>气体注射器</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>研钵和研杵</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>本生燃烧器</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>坩埚</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>输送管</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Not accurate, but fast</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Very accurate, only fixed volume</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Very accurate, variable volumes</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>More suitable for heating</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>To keep temperature constant</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>To stir, evenly mix</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Used for filtration</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Used for gas collection</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>To grind into small pieces or powder</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>Used for heating</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <t>To deliver gas</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
@@ -2176,6 +2405,12 @@
   </cellStyles>
   <dxfs count="3">
     <dxf>
+      <alignment horizontal="left" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <font>
         <b/>
         <color rgb="FFB3261E"/>
@@ -2185,12 +2420,6 @@
           <bgColor rgb="FFFCE8E6"/>
         </patternFill>
       </fill>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -2206,11 +2435,11 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="QuestionBank" displayName="QuestionBank" ref="A1:J184" totalsRowShown="0">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="QuestionBank" displayName="QuestionBank" ref="A1:J200" totalsRowShown="0">
   <tableColumns count="10">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="id"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="paper" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="topic" dataDxfId="1"/>
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="paper" dataDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="topic" dataDxfId="0"/>
     <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="question"/>
     <tableColumn id="5" xr3:uid="{00000000-0010-0000-0000-000005000000}" name="answer_1"/>
     <tableColumn id="6" xr3:uid="{00000000-0010-0000-0000-000006000000}" name="answer_2"/>
@@ -2418,7 +2647,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:J184"/>
+  <dimension ref="A1:J200"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -2468,7 +2697,7 @@
         <v>4</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>11</v>
@@ -2494,7 +2723,7 @@
         <v>4</v>
       </c>
       <c r="C3" s="7" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="D3" s="5" t="s">
         <v>16</v>
@@ -2520,7 +2749,7 @@
         <v>4</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>650</v>
+        <v>648</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>20</v>
@@ -2544,7 +2773,7 @@
         <v>4</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>23</v>
@@ -2568,7 +2797,7 @@
         <v>4</v>
       </c>
       <c r="C6" s="7" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>26</v>
@@ -2592,7 +2821,7 @@
         <v>4</v>
       </c>
       <c r="C7" s="7" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="D7" s="5" t="s">
         <v>29</v>
@@ -2616,7 +2845,7 @@
         <v>4</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="D8" s="5" t="s">
         <v>32</v>
@@ -2640,7 +2869,7 @@
         <v>4</v>
       </c>
       <c r="C9" s="7" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>35</v>
@@ -2664,7 +2893,7 @@
         <v>4</v>
       </c>
       <c r="C10" s="7" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>38</v>
@@ -2688,7 +2917,7 @@
         <v>4</v>
       </c>
       <c r="C11" s="7" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>41</v>
@@ -2714,7 +2943,7 @@
         <v>4</v>
       </c>
       <c r="C12" s="7" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="D12" s="5" t="s">
         <v>45</v>
@@ -2742,7 +2971,7 @@
         <v>4</v>
       </c>
       <c r="C13" s="7" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>50</v>
@@ -2766,7 +2995,7 @@
         <v>4</v>
       </c>
       <c r="C14" s="7" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="D14" s="5" t="s">
         <v>53</v>
@@ -2790,7 +3019,7 @@
         <v>4</v>
       </c>
       <c r="C15" s="7" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="D15" s="5" t="s">
         <v>56</v>
@@ -2814,7 +3043,7 @@
         <v>4</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="D16" s="5" t="s">
         <v>59</v>
@@ -2840,7 +3069,7 @@
         <v>4</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="D17" s="5" t="s">
         <v>63</v>
@@ -2868,7 +3097,7 @@
         <v>4</v>
       </c>
       <c r="C18" s="7" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="D18" s="5" t="s">
         <v>68</v>
@@ -2894,7 +3123,7 @@
         <v>4</v>
       </c>
       <c r="C19" s="7" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="D19" s="5" t="s">
         <v>72</v>
@@ -2920,7 +3149,7 @@
         <v>4</v>
       </c>
       <c r="C20" s="7" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>75</v>
@@ -2946,7 +3175,7 @@
         <v>4</v>
       </c>
       <c r="C21" s="7" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>79</v>
@@ -2970,7 +3199,7 @@
         <v>4</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="D22" s="5" t="s">
         <v>82</v>
@@ -2994,7 +3223,7 @@
         <v>4</v>
       </c>
       <c r="C23" s="7" t="s">
-        <v>651</v>
+        <v>649</v>
       </c>
       <c r="D23" s="5" t="s">
         <v>85</v>
@@ -3018,7 +3247,7 @@
         <v>4</v>
       </c>
       <c r="C24" s="8" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="D24" s="5" t="s">
         <v>87</v>
@@ -3046,7 +3275,7 @@
         <v>4</v>
       </c>
       <c r="C25" s="8" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="D25" s="5" t="s">
         <v>92</v>
@@ -3070,7 +3299,7 @@
         <v>4</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="D26" s="5" t="s">
         <v>95</v>
@@ -3096,7 +3325,7 @@
         <v>4</v>
       </c>
       <c r="C27" s="8" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="D27" s="5" t="s">
         <v>99</v>
@@ -3120,7 +3349,7 @@
         <v>4</v>
       </c>
       <c r="C28" s="8" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="D28" s="5" t="s">
         <v>102</v>
@@ -3144,7 +3373,7 @@
         <v>4</v>
       </c>
       <c r="C29" s="8" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="D29" s="5" t="s">
         <v>105</v>
@@ -3168,7 +3397,7 @@
         <v>4</v>
       </c>
       <c r="C30" s="8" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="D30" s="5" t="s">
         <v>108</v>
@@ -3192,7 +3421,7 @@
         <v>4</v>
       </c>
       <c r="C31" s="8" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="D31" s="5" t="s">
         <v>111</v>
@@ -3218,7 +3447,7 @@
         <v>4</v>
       </c>
       <c r="C32" s="8" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="D32" s="5" t="s">
         <v>115</v>
@@ -3242,7 +3471,7 @@
         <v>4</v>
       </c>
       <c r="C33" s="8" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="D33" s="5" t="s">
         <v>118</v>
@@ -3270,7 +3499,7 @@
         <v>4</v>
       </c>
       <c r="C34" s="8" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="D34" s="5" t="s">
         <v>123</v>
@@ -3296,7 +3525,7 @@
         <v>4</v>
       </c>
       <c r="C35" s="8" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="D35" s="5" t="s">
         <v>127</v>
@@ -3322,7 +3551,7 @@
         <v>4</v>
       </c>
       <c r="C36" s="8" t="s">
-        <v>652</v>
+        <v>650</v>
       </c>
       <c r="D36" s="5" t="s">
         <v>131</v>
@@ -3348,7 +3577,7 @@
         <v>4</v>
       </c>
       <c r="C37" s="8" t="s">
-        <v>653</v>
+        <v>651</v>
       </c>
       <c r="D37" s="5" t="s">
         <v>135</v>
@@ -3372,7 +3601,7 @@
         <v>4</v>
       </c>
       <c r="C38" s="8" t="s">
-        <v>653</v>
+        <v>651</v>
       </c>
       <c r="D38" s="5" t="s">
         <v>138</v>
@@ -3396,7 +3625,7 @@
         <v>4</v>
       </c>
       <c r="C39" s="8" t="s">
-        <v>653</v>
+        <v>651</v>
       </c>
       <c r="D39" s="5" t="s">
         <v>141</v>
@@ -3420,7 +3649,7 @@
         <v>4</v>
       </c>
       <c r="C40" s="8" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="D40" s="5" t="s">
         <v>144</v>
@@ -3444,7 +3673,7 @@
         <v>4</v>
       </c>
       <c r="C41" s="8" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="D41" s="5" t="s">
         <v>147</v>
@@ -3468,7 +3697,7 @@
         <v>4</v>
       </c>
       <c r="C42" s="8" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="D42" s="5" t="s">
         <v>150</v>
@@ -3492,7 +3721,7 @@
         <v>4</v>
       </c>
       <c r="C43" s="8" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="D43" s="5" t="s">
         <v>153</v>
@@ -3520,7 +3749,7 @@
         <v>4</v>
       </c>
       <c r="C44" s="8" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="D44" s="5" t="s">
         <v>158</v>
@@ -3546,7 +3775,7 @@
         <v>4</v>
       </c>
       <c r="C45" s="8" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="D45" s="5" t="s">
         <v>162</v>
@@ -3572,7 +3801,7 @@
         <v>4</v>
       </c>
       <c r="C46" s="8" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="D46" s="5" t="s">
         <v>165</v>
@@ -3600,7 +3829,7 @@
         <v>4</v>
       </c>
       <c r="C47" s="8" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="D47" s="5" t="s">
         <v>170</v>
@@ -3628,7 +3857,7 @@
         <v>4</v>
       </c>
       <c r="C48" s="8" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="D48" s="5" t="s">
         <v>175</v>
@@ -3652,7 +3881,7 @@
         <v>4</v>
       </c>
       <c r="C49" s="8" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="D49" s="5" t="s">
         <v>178</v>
@@ -3678,7 +3907,7 @@
         <v>4</v>
       </c>
       <c r="C50" s="8" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="D50" s="5" t="s">
         <v>182</v>
@@ -3702,7 +3931,7 @@
         <v>4</v>
       </c>
       <c r="C51" s="8" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="D51" s="5" t="s">
         <v>185</v>
@@ -3728,7 +3957,7 @@
         <v>4</v>
       </c>
       <c r="C52" s="8" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="D52" s="5" t="s">
         <v>188</v>
@@ -3756,7 +3985,7 @@
         <v>4</v>
       </c>
       <c r="C53" s="8" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="D53" s="5" t="s">
         <v>193</v>
@@ -3782,7 +4011,7 @@
         <v>4</v>
       </c>
       <c r="C54" s="8" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="D54" s="5" t="s">
         <v>197</v>
@@ -3810,7 +4039,7 @@
         <v>4</v>
       </c>
       <c r="C55" s="8" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="D55" s="5" t="s">
         <v>202</v>
@@ -3836,7 +4065,7 @@
         <v>4</v>
       </c>
       <c r="C56" s="8" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="D56" s="5" t="s">
         <v>206</v>
@@ -3864,7 +4093,7 @@
         <v>4</v>
       </c>
       <c r="C57" s="8" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="D57" s="5" t="s">
         <v>210</v>
@@ -3888,7 +4117,7 @@
         <v>4</v>
       </c>
       <c r="C58" s="8" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="D58" s="5" t="s">
         <v>213</v>
@@ -3912,7 +4141,7 @@
         <v>4</v>
       </c>
       <c r="C59" s="8" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="D59" s="5" t="s">
         <v>216</v>
@@ -3938,7 +4167,7 @@
         <v>4</v>
       </c>
       <c r="C60" s="8" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="D60" s="5" t="s">
         <v>220</v>
@@ -3964,7 +4193,7 @@
         <v>4</v>
       </c>
       <c r="C61" s="8" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="D61" s="5" t="s">
         <v>222</v>
@@ -3988,7 +4217,7 @@
         <v>4</v>
       </c>
       <c r="C62" s="8" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="D62" s="5" t="s">
         <v>225</v>
@@ -4012,7 +4241,7 @@
         <v>4</v>
       </c>
       <c r="C63" s="8" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="D63" s="5" t="s">
         <v>228</v>
@@ -4036,7 +4265,7 @@
         <v>4</v>
       </c>
       <c r="C64" s="8" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="D64" s="5" t="s">
         <v>231</v>
@@ -4060,7 +4289,7 @@
         <v>4</v>
       </c>
       <c r="C65" s="8" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="D65" s="5" t="s">
         <v>234</v>
@@ -4084,7 +4313,7 @@
         <v>4</v>
       </c>
       <c r="C66" s="8" t="s">
-        <v>654</v>
+        <v>652</v>
       </c>
       <c r="D66" s="5" t="s">
         <v>237</v>
@@ -4108,7 +4337,7 @@
         <v>4</v>
       </c>
       <c r="C67" s="8" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="D67" s="5" t="s">
         <v>240</v>
@@ -4134,7 +4363,7 @@
         <v>4</v>
       </c>
       <c r="C68" s="8" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="D68" s="5" t="s">
         <v>244</v>
@@ -4158,7 +4387,7 @@
         <v>4</v>
       </c>
       <c r="C69" s="8" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="D69" s="5" t="s">
         <v>247</v>
@@ -4182,7 +4411,7 @@
         <v>4</v>
       </c>
       <c r="C70" s="8" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="D70" s="5" t="s">
         <v>250</v>
@@ -4206,7 +4435,7 @@
         <v>4</v>
       </c>
       <c r="C71" s="8" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="D71" s="5" t="s">
         <v>253</v>
@@ -4230,7 +4459,7 @@
         <v>4</v>
       </c>
       <c r="C72" s="8" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="D72" s="5" t="s">
         <v>256</v>
@@ -4254,7 +4483,7 @@
         <v>4</v>
       </c>
       <c r="C73" s="8" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="D73" s="5" t="s">
         <v>259</v>
@@ -4278,7 +4507,7 @@
         <v>4</v>
       </c>
       <c r="C74" s="8" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="D74" s="5" t="s">
         <v>262</v>
@@ -4302,7 +4531,7 @@
         <v>4</v>
       </c>
       <c r="C75" s="8" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="D75" s="5" t="s">
         <v>265</v>
@@ -4326,7 +4555,7 @@
         <v>4</v>
       </c>
       <c r="C76" s="8" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="D76" s="5" t="s">
         <v>268</v>
@@ -4350,7 +4579,7 @@
         <v>4</v>
       </c>
       <c r="C77" s="8" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="D77" s="5" t="s">
         <v>271</v>
@@ -4374,7 +4603,7 @@
         <v>4</v>
       </c>
       <c r="C78" s="8" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="D78" s="5" t="s">
         <v>274</v>
@@ -4406,7 +4635,7 @@
         <v>4</v>
       </c>
       <c r="C79" s="8" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="D79" s="5" t="s">
         <v>281</v>
@@ -4432,7 +4661,7 @@
         <v>4</v>
       </c>
       <c r="C80" s="8" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="D80" s="5" t="s">
         <v>285</v>
@@ -4456,7 +4685,7 @@
         <v>4</v>
       </c>
       <c r="C81" s="8" t="s">
-        <v>655</v>
+        <v>653</v>
       </c>
       <c r="D81" s="5" t="s">
         <v>288</v>
@@ -4484,7 +4713,7 @@
         <v>4</v>
       </c>
       <c r="C82" s="8" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="D82" s="5" t="s">
         <v>292</v>
@@ -4508,7 +4737,7 @@
         <v>4</v>
       </c>
       <c r="C83" s="8" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="D83" s="5" t="s">
         <v>295</v>
@@ -4532,7 +4761,7 @@
         <v>4</v>
       </c>
       <c r="C84" s="8" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="D84" s="5" t="s">
         <v>298</v>
@@ -4556,7 +4785,7 @@
         <v>4</v>
       </c>
       <c r="C85" s="8" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="D85" s="5" t="s">
         <v>300</v>
@@ -4580,7 +4809,7 @@
         <v>4</v>
       </c>
       <c r="C86" s="8" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="D86" s="5" t="s">
         <v>303</v>
@@ -4610,7 +4839,7 @@
         <v>4</v>
       </c>
       <c r="C87" s="8" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="D87" s="5" t="s">
         <v>309</v>
@@ -4638,7 +4867,7 @@
         <v>4</v>
       </c>
       <c r="C88" s="8" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="D88" s="5" t="s">
         <v>314</v>
@@ -4666,7 +4895,7 @@
         <v>4</v>
       </c>
       <c r="C89" s="8" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="D89" s="5" t="s">
         <v>319</v>
@@ -4690,7 +4919,7 @@
         <v>4</v>
       </c>
       <c r="C90" s="8" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="D90" s="5" t="s">
         <v>322</v>
@@ -4714,7 +4943,7 @@
         <v>4</v>
       </c>
       <c r="C91" s="8" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="D91" s="5" t="s">
         <v>325</v>
@@ -4744,7 +4973,7 @@
         <v>4</v>
       </c>
       <c r="C92" s="8" t="s">
-        <v>656</v>
+        <v>654</v>
       </c>
       <c r="D92" s="5" t="s">
         <v>331</v>
@@ -4768,7 +4997,7 @@
         <v>4</v>
       </c>
       <c r="C93" s="8" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="D93" s="5" t="s">
         <v>334</v>
@@ -4794,7 +5023,7 @@
         <v>4</v>
       </c>
       <c r="C94" s="8" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="D94" s="5" t="s">
         <v>338</v>
@@ -4820,7 +5049,7 @@
         <v>4</v>
       </c>
       <c r="C95" s="8" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="D95" s="5" t="s">
         <v>342</v>
@@ -4844,7 +5073,7 @@
         <v>4</v>
       </c>
       <c r="C96" s="8" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="D96" s="5" t="s">
         <v>345</v>
@@ -4868,7 +5097,7 @@
         <v>4</v>
       </c>
       <c r="C97" s="8" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="D97" s="5" t="s">
         <v>348</v>
@@ -4894,7 +5123,7 @@
         <v>4</v>
       </c>
       <c r="C98" s="8" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="D98" s="5" t="s">
         <v>352</v>
@@ -4918,7 +5147,7 @@
         <v>4</v>
       </c>
       <c r="C99" s="8" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="D99" s="5" t="s">
         <v>355</v>
@@ -4942,7 +5171,7 @@
         <v>4</v>
       </c>
       <c r="C100" s="8" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="D100" s="5" t="s">
         <v>358</v>
@@ -4968,7 +5197,7 @@
         <v>4</v>
       </c>
       <c r="C101" s="8" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="D101" s="5" t="s">
         <v>362</v>
@@ -4992,7 +5221,7 @@
         <v>4</v>
       </c>
       <c r="C102" s="8" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="D102" s="5" t="s">
         <v>365</v>
@@ -5018,7 +5247,7 @@
         <v>4</v>
       </c>
       <c r="C103" s="8" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="D103" s="5" t="s">
         <v>369</v>
@@ -5042,7 +5271,7 @@
         <v>4</v>
       </c>
       <c r="C104" s="8" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="D104" s="5" t="s">
         <v>372</v>
@@ -5066,7 +5295,7 @@
         <v>4</v>
       </c>
       <c r="C105" s="8" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="D105" s="5" t="s">
         <v>375</v>
@@ -5094,7 +5323,7 @@
         <v>4</v>
       </c>
       <c r="C106" s="8" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="D106" s="5" t="s">
         <v>380</v>
@@ -5118,7 +5347,7 @@
         <v>4</v>
       </c>
       <c r="C107" s="8" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="D107" s="5" t="s">
         <v>383</v>
@@ -5142,7 +5371,7 @@
         <v>4</v>
       </c>
       <c r="C108" s="8" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="D108" s="5" t="s">
         <v>386</v>
@@ -5166,7 +5395,7 @@
         <v>4</v>
       </c>
       <c r="C109" s="8" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="D109" s="5" t="s">
         <v>389</v>
@@ -5190,7 +5419,7 @@
         <v>4</v>
       </c>
       <c r="C110" s="8" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="D110" s="5" t="s">
         <v>392</v>
@@ -5218,7 +5447,7 @@
         <v>4</v>
       </c>
       <c r="C111" s="8" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="D111" s="5" t="s">
         <v>397</v>
@@ -5242,7 +5471,7 @@
         <v>4</v>
       </c>
       <c r="C112" s="8" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="D112" s="5" t="s">
         <v>400</v>
@@ -5266,7 +5495,7 @@
         <v>4</v>
       </c>
       <c r="C113" s="8" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="D113" s="5" t="s">
         <v>403</v>
@@ -5294,7 +5523,7 @@
         <v>4</v>
       </c>
       <c r="C114" s="8" t="s">
-        <v>657</v>
+        <v>655</v>
       </c>
       <c r="D114" s="5" t="s">
         <v>408</v>
@@ -5318,7 +5547,7 @@
         <v>4</v>
       </c>
       <c r="C115" s="8" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="D115" s="5" t="s">
         <v>411</v>
@@ -5344,7 +5573,7 @@
         <v>4</v>
       </c>
       <c r="C116" s="8" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="D116" s="5" t="s">
         <v>415</v>
@@ -5368,7 +5597,7 @@
         <v>4</v>
       </c>
       <c r="C117" s="8" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="D117" s="5" t="s">
         <v>418</v>
@@ -5392,7 +5621,7 @@
         <v>4</v>
       </c>
       <c r="C118" s="8" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="D118" s="5" t="s">
         <v>421</v>
@@ -5422,7 +5651,7 @@
         <v>4</v>
       </c>
       <c r="C119" s="8" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="D119" s="5" t="s">
         <v>427</v>
@@ -5446,7 +5675,7 @@
         <v>4</v>
       </c>
       <c r="C120" s="8" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="D120" s="5" t="s">
         <v>430</v>
@@ -5470,7 +5699,7 @@
         <v>4</v>
       </c>
       <c r="C121" s="8" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="D121" s="5" t="s">
         <v>433</v>
@@ -5500,7 +5729,7 @@
         <v>4</v>
       </c>
       <c r="C122" s="8" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="D122" s="5" t="s">
         <v>438</v>
@@ -5526,7 +5755,7 @@
         <v>4</v>
       </c>
       <c r="C123" s="8" t="s">
-        <v>658</v>
+        <v>656</v>
       </c>
       <c r="D123" s="5" t="s">
         <v>442</v>
@@ -5550,7 +5779,7 @@
         <v>4</v>
       </c>
       <c r="C124" s="8" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="D124" s="5" t="s">
         <v>445</v>
@@ -5574,7 +5803,7 @@
         <v>4</v>
       </c>
       <c r="C125" s="8" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="D125" s="5" t="s">
         <v>448</v>
@@ -5598,7 +5827,7 @@
         <v>4</v>
       </c>
       <c r="C126" s="8" t="s">
-        <v>659</v>
+        <v>657</v>
       </c>
       <c r="D126" s="5" t="s">
         <v>451</v>
@@ -5610,13 +5839,13 @@
         <v>453</v>
       </c>
       <c r="G126" s="5" t="s">
+        <v>664</v>
+      </c>
+      <c r="H126" s="5" t="s">
         <v>454</v>
       </c>
-      <c r="H126" s="5" t="s">
+      <c r="I126" s="5" t="s">
         <v>455</v>
-      </c>
-      <c r="I126" s="5" t="s">
-        <v>456</v>
       </c>
       <c r="J126" s="5" t="s">
         <v>14</v>
@@ -5624,19 +5853,19 @@
     </row>
     <row r="127" spans="1:10" ht="42" customHeight="1">
       <c r="A127" s="4" t="s">
+        <v>456</v>
+      </c>
+      <c r="B127" s="8">
+        <v>4</v>
+      </c>
+      <c r="C127" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="D127" s="5" t="s">
         <v>457</v>
       </c>
-      <c r="B127" s="8">
-        <v>4</v>
-      </c>
-      <c r="C127" s="8" t="s">
-        <v>659</v>
-      </c>
-      <c r="D127" s="5" t="s">
+      <c r="E127" s="5" t="s">
         <v>458</v>
-      </c>
-      <c r="E127" s="5" t="s">
-        <v>459</v>
       </c>
       <c r="F127" s="5"/>
       <c r="G127" s="5"/>
@@ -5648,19 +5877,19 @@
     </row>
     <row r="128" spans="1:10" ht="42" customHeight="1">
       <c r="A128" s="4" t="s">
+        <v>459</v>
+      </c>
+      <c r="B128" s="8">
+        <v>4</v>
+      </c>
+      <c r="C128" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="D128" s="5" t="s">
         <v>460</v>
       </c>
-      <c r="B128" s="8">
-        <v>4</v>
-      </c>
-      <c r="C128" s="8" t="s">
-        <v>659</v>
-      </c>
-      <c r="D128" s="5" t="s">
+      <c r="E128" s="5" t="s">
         <v>461</v>
-      </c>
-      <c r="E128" s="5" t="s">
-        <v>462</v>
       </c>
       <c r="F128" s="5"/>
       <c r="G128" s="5"/>
@@ -5672,22 +5901,22 @@
     </row>
     <row r="129" spans="1:10" ht="42" customHeight="1">
       <c r="A129" s="4" t="s">
+        <v>462</v>
+      </c>
+      <c r="B129" s="8">
+        <v>4</v>
+      </c>
+      <c r="C129" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="D129" s="5" t="s">
         <v>463</v>
       </c>
-      <c r="B129" s="8">
-        <v>4</v>
-      </c>
-      <c r="C129" s="8" t="s">
-        <v>659</v>
-      </c>
-      <c r="D129" s="5" t="s">
+      <c r="E129" s="5" t="s">
         <v>464</v>
       </c>
-      <c r="E129" s="5" t="s">
+      <c r="F129" s="5" t="s">
         <v>465</v>
-      </c>
-      <c r="F129" s="5" t="s">
-        <v>466</v>
       </c>
       <c r="G129" s="5"/>
       <c r="H129" s="5"/>
@@ -5698,19 +5927,19 @@
     </row>
     <row r="130" spans="1:10" ht="42" customHeight="1">
       <c r="A130" s="4" t="s">
+        <v>466</v>
+      </c>
+      <c r="B130" s="7">
+        <v>4</v>
+      </c>
+      <c r="C130" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="D130" s="5" t="s">
         <v>467</v>
       </c>
-      <c r="B130" s="7">
-        <v>4</v>
-      </c>
-      <c r="C130" s="8" t="s">
-        <v>659</v>
-      </c>
-      <c r="D130" s="5" t="s">
+      <c r="E130" s="5" t="s">
         <v>468</v>
-      </c>
-      <c r="E130" s="5" t="s">
-        <v>469</v>
       </c>
       <c r="F130" s="5"/>
       <c r="G130" s="5"/>
@@ -5722,19 +5951,19 @@
     </row>
     <row r="131" spans="1:10" ht="42" customHeight="1">
       <c r="A131" s="4" t="s">
+        <v>469</v>
+      </c>
+      <c r="B131" s="8">
+        <v>4</v>
+      </c>
+      <c r="C131" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="D131" s="5" t="s">
         <v>470</v>
       </c>
-      <c r="B131" s="8">
-        <v>4</v>
-      </c>
-      <c r="C131" s="8" t="s">
-        <v>659</v>
-      </c>
-      <c r="D131" s="5" t="s">
+      <c r="E131" s="5" t="s">
         <v>471</v>
-      </c>
-      <c r="E131" s="5" t="s">
-        <v>472</v>
       </c>
       <c r="F131" s="5"/>
       <c r="G131" s="5"/>
@@ -5746,19 +5975,19 @@
     </row>
     <row r="132" spans="1:10" ht="42" customHeight="1">
       <c r="A132" s="4" t="s">
+        <v>472</v>
+      </c>
+      <c r="B132" s="8">
+        <v>4</v>
+      </c>
+      <c r="C132" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="D132" s="5" t="s">
         <v>473</v>
       </c>
-      <c r="B132" s="8">
-        <v>4</v>
-      </c>
-      <c r="C132" s="8" t="s">
-        <v>659</v>
-      </c>
-      <c r="D132" s="5" t="s">
+      <c r="E132" s="5" t="s">
         <v>474</v>
-      </c>
-      <c r="E132" s="5" t="s">
-        <v>475</v>
       </c>
       <c r="F132" s="5"/>
       <c r="G132" s="5"/>
@@ -5770,19 +5999,19 @@
     </row>
     <row r="133" spans="1:10" ht="42" customHeight="1">
       <c r="A133" s="4" t="s">
+        <v>475</v>
+      </c>
+      <c r="B133" s="8">
+        <v>4</v>
+      </c>
+      <c r="C133" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="D133" s="5" t="s">
         <v>476</v>
       </c>
-      <c r="B133" s="8">
-        <v>4</v>
-      </c>
-      <c r="C133" s="8" t="s">
-        <v>659</v>
-      </c>
-      <c r="D133" s="5" t="s">
+      <c r="E133" s="5" t="s">
         <v>477</v>
-      </c>
-      <c r="E133" s="5" t="s">
-        <v>478</v>
       </c>
       <c r="F133" s="5"/>
       <c r="G133" s="5"/>
@@ -5794,19 +6023,19 @@
     </row>
     <row r="134" spans="1:10" ht="42" customHeight="1">
       <c r="A134" s="4" t="s">
+        <v>478</v>
+      </c>
+      <c r="B134" s="7">
+        <v>4</v>
+      </c>
+      <c r="C134" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="D134" s="5" t="s">
         <v>479</v>
       </c>
-      <c r="B134" s="7">
-        <v>4</v>
-      </c>
-      <c r="C134" s="8" t="s">
-        <v>659</v>
-      </c>
-      <c r="D134" s="5" t="s">
+      <c r="E134" s="5" t="s">
         <v>480</v>
-      </c>
-      <c r="E134" s="5" t="s">
-        <v>481</v>
       </c>
       <c r="F134" s="5"/>
       <c r="G134" s="5"/>
@@ -5818,22 +6047,22 @@
     </row>
     <row r="135" spans="1:10" ht="42" customHeight="1">
       <c r="A135" s="4" t="s">
+        <v>481</v>
+      </c>
+      <c r="B135" s="8">
+        <v>4</v>
+      </c>
+      <c r="C135" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="D135" s="5" t="s">
         <v>482</v>
       </c>
-      <c r="B135" s="8">
-        <v>4</v>
-      </c>
-      <c r="C135" s="8" t="s">
-        <v>659</v>
-      </c>
-      <c r="D135" s="5" t="s">
+      <c r="E135" s="5" t="s">
         <v>483</v>
       </c>
-      <c r="E135" s="5" t="s">
-        <v>484</v>
-      </c>
       <c r="F135" s="5" t="s">
-        <v>485</v>
+        <v>663</v>
       </c>
       <c r="G135" s="5"/>
       <c r="H135" s="5"/>
@@ -5844,19 +6073,19 @@
     </row>
     <row r="136" spans="1:10" ht="42" customHeight="1">
       <c r="A136" s="4" t="s">
+        <v>484</v>
+      </c>
+      <c r="B136" s="8">
+        <v>4</v>
+      </c>
+      <c r="C136" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="D136" s="5" t="s">
+        <v>485</v>
+      </c>
+      <c r="E136" s="5" t="s">
         <v>486</v>
-      </c>
-      <c r="B136" s="8">
-        <v>4</v>
-      </c>
-      <c r="C136" s="8" t="s">
-        <v>659</v>
-      </c>
-      <c r="D136" s="5" t="s">
-        <v>487</v>
-      </c>
-      <c r="E136" s="5" t="s">
-        <v>488</v>
       </c>
       <c r="F136" s="5"/>
       <c r="G136" s="5"/>
@@ -5868,19 +6097,19 @@
     </row>
     <row r="137" spans="1:10" ht="42" customHeight="1">
       <c r="A137" s="4" t="s">
+        <v>487</v>
+      </c>
+      <c r="B137" s="8">
+        <v>4</v>
+      </c>
+      <c r="C137" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="D137" s="5" t="s">
+        <v>488</v>
+      </c>
+      <c r="E137" s="5" t="s">
         <v>489</v>
-      </c>
-      <c r="B137" s="8">
-        <v>4</v>
-      </c>
-      <c r="C137" s="8" t="s">
-        <v>659</v>
-      </c>
-      <c r="D137" s="5" t="s">
-        <v>490</v>
-      </c>
-      <c r="E137" s="5" t="s">
-        <v>491</v>
       </c>
       <c r="F137" s="5"/>
       <c r="G137" s="5"/>
@@ -5892,25 +6121,25 @@
     </row>
     <row r="138" spans="1:10" ht="42" customHeight="1">
       <c r="A138" s="4" t="s">
+        <v>490</v>
+      </c>
+      <c r="B138" s="7">
+        <v>4</v>
+      </c>
+      <c r="C138" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="D138" s="5" t="s">
+        <v>491</v>
+      </c>
+      <c r="E138" s="5" t="s">
         <v>492</v>
       </c>
-      <c r="B138" s="7">
-        <v>4</v>
-      </c>
-      <c r="C138" s="8" t="s">
-        <v>659</v>
-      </c>
-      <c r="D138" s="5" t="s">
+      <c r="F138" s="5" t="s">
         <v>493</v>
       </c>
-      <c r="E138" s="5" t="s">
+      <c r="G138" s="5" t="s">
         <v>494</v>
-      </c>
-      <c r="F138" s="5" t="s">
-        <v>495</v>
-      </c>
-      <c r="G138" s="5" t="s">
-        <v>496</v>
       </c>
       <c r="H138" s="5"/>
       <c r="I138" s="5"/>
@@ -5920,22 +6149,22 @@
     </row>
     <row r="139" spans="1:10" ht="42" customHeight="1">
       <c r="A139" s="4" t="s">
+        <v>495</v>
+      </c>
+      <c r="B139" s="8">
+        <v>4</v>
+      </c>
+      <c r="C139" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="D139" s="5" t="s">
+        <v>496</v>
+      </c>
+      <c r="E139" s="5" t="s">
         <v>497</v>
       </c>
-      <c r="B139" s="8">
-        <v>4</v>
-      </c>
-      <c r="C139" s="8" t="s">
-        <v>659</v>
-      </c>
-      <c r="D139" s="5" t="s">
+      <c r="F139" s="5" t="s">
         <v>498</v>
-      </c>
-      <c r="E139" s="5" t="s">
-        <v>499</v>
-      </c>
-      <c r="F139" s="5" t="s">
-        <v>500</v>
       </c>
       <c r="G139" s="5"/>
       <c r="H139" s="5"/>
@@ -5946,22 +6175,22 @@
     </row>
     <row r="140" spans="1:10" ht="42" customHeight="1">
       <c r="A140" s="4" t="s">
+        <v>499</v>
+      </c>
+      <c r="B140" s="8">
+        <v>4</v>
+      </c>
+      <c r="C140" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="D140" s="5" t="s">
+        <v>500</v>
+      </c>
+      <c r="E140" s="5" t="s">
         <v>501</v>
       </c>
-      <c r="B140" s="8">
-        <v>4</v>
-      </c>
-      <c r="C140" s="8" t="s">
-        <v>659</v>
-      </c>
-      <c r="D140" s="5" t="s">
+      <c r="F140" s="5" t="s">
         <v>502</v>
-      </c>
-      <c r="E140" s="5" t="s">
-        <v>503</v>
-      </c>
-      <c r="F140" s="5" t="s">
-        <v>504</v>
       </c>
       <c r="G140" s="5"/>
       <c r="H140" s="5"/>
@@ -5972,25 +6201,25 @@
     </row>
     <row r="141" spans="1:10" ht="42" customHeight="1">
       <c r="A141" s="4" t="s">
+        <v>503</v>
+      </c>
+      <c r="B141" s="8">
+        <v>4</v>
+      </c>
+      <c r="C141" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="D141" s="5" t="s">
+        <v>504</v>
+      </c>
+      <c r="E141" s="5" t="s">
         <v>505</v>
       </c>
-      <c r="B141" s="8">
-        <v>4</v>
-      </c>
-      <c r="C141" s="8" t="s">
-        <v>659</v>
-      </c>
-      <c r="D141" s="5" t="s">
+      <c r="F141" s="5" t="s">
         <v>506</v>
       </c>
-      <c r="E141" s="5" t="s">
+      <c r="G141" s="5" t="s">
         <v>507</v>
-      </c>
-      <c r="F141" s="5" t="s">
-        <v>508</v>
-      </c>
-      <c r="G141" s="5" t="s">
-        <v>509</v>
       </c>
       <c r="H141" s="5"/>
       <c r="I141" s="5"/>
@@ -6000,22 +6229,22 @@
     </row>
     <row r="142" spans="1:10" ht="42" customHeight="1">
       <c r="A142" s="4" t="s">
+        <v>508</v>
+      </c>
+      <c r="B142" s="7">
+        <v>4</v>
+      </c>
+      <c r="C142" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="D142" s="5" t="s">
+        <v>509</v>
+      </c>
+      <c r="E142" s="5" t="s">
         <v>510</v>
       </c>
-      <c r="B142" s="7">
-        <v>4</v>
-      </c>
-      <c r="C142" s="8" t="s">
-        <v>659</v>
-      </c>
-      <c r="D142" s="5" t="s">
+      <c r="F142" s="5" t="s">
         <v>511</v>
-      </c>
-      <c r="E142" s="5" t="s">
-        <v>512</v>
-      </c>
-      <c r="F142" s="5" t="s">
-        <v>513</v>
       </c>
       <c r="G142" s="5"/>
       <c r="H142" s="5"/>
@@ -6026,22 +6255,22 @@
     </row>
     <row r="143" spans="1:10" ht="42" customHeight="1">
       <c r="A143" s="4" t="s">
+        <v>512</v>
+      </c>
+      <c r="B143" s="8">
+        <v>4</v>
+      </c>
+      <c r="C143" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="D143" s="5" t="s">
+        <v>513</v>
+      </c>
+      <c r="E143" s="5" t="s">
         <v>514</v>
       </c>
-      <c r="B143" s="8">
-        <v>4</v>
-      </c>
-      <c r="C143" s="8" t="s">
-        <v>659</v>
-      </c>
-      <c r="D143" s="5" t="s">
+      <c r="F143" s="5" t="s">
         <v>515</v>
-      </c>
-      <c r="E143" s="5" t="s">
-        <v>516</v>
-      </c>
-      <c r="F143" s="5" t="s">
-        <v>517</v>
       </c>
       <c r="G143" s="5"/>
       <c r="H143" s="5"/>
@@ -6052,19 +6281,19 @@
     </row>
     <row r="144" spans="1:10" ht="42" customHeight="1">
       <c r="A144" s="4" t="s">
+        <v>516</v>
+      </c>
+      <c r="B144" s="8">
+        <v>4</v>
+      </c>
+      <c r="C144" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="D144" s="5" t="s">
+        <v>517</v>
+      </c>
+      <c r="E144" s="5" t="s">
         <v>518</v>
-      </c>
-      <c r="B144" s="8">
-        <v>4</v>
-      </c>
-      <c r="C144" s="8" t="s">
-        <v>659</v>
-      </c>
-      <c r="D144" s="5" t="s">
-        <v>519</v>
-      </c>
-      <c r="E144" s="5" t="s">
-        <v>520</v>
       </c>
       <c r="F144" s="5"/>
       <c r="G144" s="5"/>
@@ -6076,19 +6305,19 @@
     </row>
     <row r="145" spans="1:10" ht="42" customHeight="1">
       <c r="A145" s="4" t="s">
+        <v>519</v>
+      </c>
+      <c r="B145" s="8">
+        <v>4</v>
+      </c>
+      <c r="C145" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="D145" s="5" t="s">
+        <v>520</v>
+      </c>
+      <c r="E145" s="5" t="s">
         <v>521</v>
-      </c>
-      <c r="B145" s="8">
-        <v>4</v>
-      </c>
-      <c r="C145" s="8" t="s">
-        <v>659</v>
-      </c>
-      <c r="D145" s="5" t="s">
-        <v>522</v>
-      </c>
-      <c r="E145" s="5" t="s">
-        <v>523</v>
       </c>
       <c r="F145" s="5"/>
       <c r="G145" s="5"/>
@@ -6100,19 +6329,19 @@
     </row>
     <row r="146" spans="1:10" ht="42" customHeight="1">
       <c r="A146" s="4" t="s">
+        <v>522</v>
+      </c>
+      <c r="B146" s="7">
+        <v>4</v>
+      </c>
+      <c r="C146" s="8" t="s">
+        <v>657</v>
+      </c>
+      <c r="D146" s="5" t="s">
+        <v>523</v>
+      </c>
+      <c r="E146" s="5" t="s">
         <v>524</v>
-      </c>
-      <c r="B146" s="7">
-        <v>4</v>
-      </c>
-      <c r="C146" s="8" t="s">
-        <v>659</v>
-      </c>
-      <c r="D146" s="5" t="s">
-        <v>525</v>
-      </c>
-      <c r="E146" s="5" t="s">
-        <v>526</v>
       </c>
       <c r="F146" s="5"/>
       <c r="G146" s="5"/>
@@ -6124,19 +6353,19 @@
     </row>
     <row r="147" spans="1:10" ht="42" customHeight="1">
       <c r="A147" s="4" t="s">
+        <v>525</v>
+      </c>
+      <c r="B147" s="8">
+        <v>4</v>
+      </c>
+      <c r="C147" s="8" t="s">
+        <v>658</v>
+      </c>
+      <c r="D147" s="5" t="s">
+        <v>526</v>
+      </c>
+      <c r="E147" s="5" t="s">
         <v>527</v>
-      </c>
-      <c r="B147" s="8">
-        <v>4</v>
-      </c>
-      <c r="C147" s="8" t="s">
-        <v>660</v>
-      </c>
-      <c r="D147" s="5" t="s">
-        <v>528</v>
-      </c>
-      <c r="E147" s="5" t="s">
-        <v>529</v>
       </c>
       <c r="F147" s="5"/>
       <c r="G147" s="5"/>
@@ -6148,19 +6377,19 @@
     </row>
     <row r="148" spans="1:10" ht="42" customHeight="1">
       <c r="A148" s="4" t="s">
+        <v>528</v>
+      </c>
+      <c r="B148" s="8">
+        <v>4</v>
+      </c>
+      <c r="C148" s="8" t="s">
+        <v>658</v>
+      </c>
+      <c r="D148" s="5" t="s">
+        <v>529</v>
+      </c>
+      <c r="E148" s="5" t="s">
         <v>530</v>
-      </c>
-      <c r="B148" s="8">
-        <v>4</v>
-      </c>
-      <c r="C148" s="8" t="s">
-        <v>660</v>
-      </c>
-      <c r="D148" s="5" t="s">
-        <v>531</v>
-      </c>
-      <c r="E148" s="5" t="s">
-        <v>532</v>
       </c>
       <c r="F148" s="5"/>
       <c r="G148" s="5"/>
@@ -6172,19 +6401,19 @@
     </row>
     <row r="149" spans="1:10" ht="42" customHeight="1">
       <c r="A149" s="4" t="s">
+        <v>531</v>
+      </c>
+      <c r="B149" s="8">
+        <v>4</v>
+      </c>
+      <c r="C149" s="8" t="s">
+        <v>658</v>
+      </c>
+      <c r="D149" s="5" t="s">
+        <v>532</v>
+      </c>
+      <c r="E149" s="5" t="s">
         <v>533</v>
-      </c>
-      <c r="B149" s="8">
-        <v>4</v>
-      </c>
-      <c r="C149" s="8" t="s">
-        <v>660</v>
-      </c>
-      <c r="D149" s="5" t="s">
-        <v>534</v>
-      </c>
-      <c r="E149" s="5" t="s">
-        <v>535</v>
       </c>
       <c r="F149" s="5"/>
       <c r="G149" s="5"/>
@@ -6196,19 +6425,19 @@
     </row>
     <row r="150" spans="1:10" ht="42" customHeight="1">
       <c r="A150" s="4" t="s">
+        <v>534</v>
+      </c>
+      <c r="B150" s="7">
+        <v>4</v>
+      </c>
+      <c r="C150" s="8" t="s">
+        <v>658</v>
+      </c>
+      <c r="D150" s="5" t="s">
+        <v>535</v>
+      </c>
+      <c r="E150" s="5" t="s">
         <v>536</v>
-      </c>
-      <c r="B150" s="7">
-        <v>4</v>
-      </c>
-      <c r="C150" s="8" t="s">
-        <v>660</v>
-      </c>
-      <c r="D150" s="5" t="s">
-        <v>537</v>
-      </c>
-      <c r="E150" s="5" t="s">
-        <v>538</v>
       </c>
       <c r="F150" s="5"/>
       <c r="G150" s="5"/>
@@ -6220,19 +6449,19 @@
     </row>
     <row r="151" spans="1:10" ht="42" customHeight="1">
       <c r="A151" s="4" t="s">
+        <v>537</v>
+      </c>
+      <c r="B151" s="8">
+        <v>4</v>
+      </c>
+      <c r="C151" s="8" t="s">
+        <v>658</v>
+      </c>
+      <c r="D151" s="5" t="s">
+        <v>538</v>
+      </c>
+      <c r="E151" s="5" t="s">
         <v>539</v>
-      </c>
-      <c r="B151" s="8">
-        <v>4</v>
-      </c>
-      <c r="C151" s="8" t="s">
-        <v>660</v>
-      </c>
-      <c r="D151" s="5" t="s">
-        <v>540</v>
-      </c>
-      <c r="E151" s="5" t="s">
-        <v>541</v>
       </c>
       <c r="F151" s="5"/>
       <c r="G151" s="5"/>
@@ -6244,19 +6473,19 @@
     </row>
     <row r="152" spans="1:10" ht="42" customHeight="1">
       <c r="A152" s="4" t="s">
+        <v>540</v>
+      </c>
+      <c r="B152" s="8">
+        <v>4</v>
+      </c>
+      <c r="C152" s="8" t="s">
+        <v>658</v>
+      </c>
+      <c r="D152" s="5" t="s">
+        <v>541</v>
+      </c>
+      <c r="E152" s="5" t="s">
         <v>542</v>
-      </c>
-      <c r="B152" s="8">
-        <v>4</v>
-      </c>
-      <c r="C152" s="8" t="s">
-        <v>660</v>
-      </c>
-      <c r="D152" s="5" t="s">
-        <v>543</v>
-      </c>
-      <c r="E152" s="5" t="s">
-        <v>544</v>
       </c>
       <c r="F152" s="5"/>
       <c r="G152" s="5"/>
@@ -6268,22 +6497,22 @@
     </row>
     <row r="153" spans="1:10" ht="42" customHeight="1">
       <c r="A153" s="4" t="s">
+        <v>543</v>
+      </c>
+      <c r="B153" s="8">
+        <v>4</v>
+      </c>
+      <c r="C153" s="8" t="s">
+        <v>658</v>
+      </c>
+      <c r="D153" s="5" t="s">
+        <v>544</v>
+      </c>
+      <c r="E153" s="5" t="s">
         <v>545</v>
       </c>
-      <c r="B153" s="8">
-        <v>4</v>
-      </c>
-      <c r="C153" s="8" t="s">
-        <v>660</v>
-      </c>
-      <c r="D153" s="5" t="s">
+      <c r="F153" s="5" t="s">
         <v>546</v>
-      </c>
-      <c r="E153" s="5" t="s">
-        <v>547</v>
-      </c>
-      <c r="F153" s="5" t="s">
-        <v>548</v>
       </c>
       <c r="G153" s="5" t="s">
         <v>279</v>
@@ -6296,19 +6525,19 @@
     </row>
     <row r="154" spans="1:10" ht="42" customHeight="1">
       <c r="A154" s="4" t="s">
+        <v>547</v>
+      </c>
+      <c r="B154" s="7">
+        <v>4</v>
+      </c>
+      <c r="C154" s="8" t="s">
+        <v>658</v>
+      </c>
+      <c r="D154" s="5" t="s">
+        <v>548</v>
+      </c>
+      <c r="E154" s="5" t="s">
         <v>549</v>
-      </c>
-      <c r="B154" s="7">
-        <v>4</v>
-      </c>
-      <c r="C154" s="8" t="s">
-        <v>660</v>
-      </c>
-      <c r="D154" s="5" t="s">
-        <v>550</v>
-      </c>
-      <c r="E154" s="5" t="s">
-        <v>551</v>
       </c>
       <c r="F154" s="5"/>
       <c r="G154" s="5"/>
@@ -6320,19 +6549,19 @@
     </row>
     <row r="155" spans="1:10" ht="42" customHeight="1">
       <c r="A155" s="4" t="s">
+        <v>550</v>
+      </c>
+      <c r="B155" s="8">
+        <v>4</v>
+      </c>
+      <c r="C155" s="8" t="s">
+        <v>658</v>
+      </c>
+      <c r="D155" s="5" t="s">
+        <v>551</v>
+      </c>
+      <c r="E155" s="5" t="s">
         <v>552</v>
-      </c>
-      <c r="B155" s="8">
-        <v>4</v>
-      </c>
-      <c r="C155" s="8" t="s">
-        <v>660</v>
-      </c>
-      <c r="D155" s="5" t="s">
-        <v>553</v>
-      </c>
-      <c r="E155" s="5" t="s">
-        <v>554</v>
       </c>
       <c r="F155" s="5"/>
       <c r="G155" s="5"/>
@@ -6344,19 +6573,19 @@
     </row>
     <row r="156" spans="1:10" ht="42" customHeight="1">
       <c r="A156" s="4" t="s">
+        <v>553</v>
+      </c>
+      <c r="B156" s="8">
+        <v>4</v>
+      </c>
+      <c r="C156" s="8" t="s">
+        <v>658</v>
+      </c>
+      <c r="D156" s="5" t="s">
+        <v>554</v>
+      </c>
+      <c r="E156" s="5" t="s">
         <v>555</v>
-      </c>
-      <c r="B156" s="8">
-        <v>4</v>
-      </c>
-      <c r="C156" s="8" t="s">
-        <v>660</v>
-      </c>
-      <c r="D156" s="5" t="s">
-        <v>556</v>
-      </c>
-      <c r="E156" s="5" t="s">
-        <v>557</v>
       </c>
       <c r="F156" s="5"/>
       <c r="G156" s="5"/>
@@ -6368,19 +6597,19 @@
     </row>
     <row r="157" spans="1:10" ht="42" customHeight="1">
       <c r="A157" s="4" t="s">
+        <v>556</v>
+      </c>
+      <c r="B157" s="8">
+        <v>4</v>
+      </c>
+      <c r="C157" s="8" t="s">
+        <v>658</v>
+      </c>
+      <c r="D157" s="5" t="s">
+        <v>557</v>
+      </c>
+      <c r="E157" s="5" t="s">
         <v>558</v>
-      </c>
-      <c r="B157" s="8">
-        <v>4</v>
-      </c>
-      <c r="C157" s="8" t="s">
-        <v>660</v>
-      </c>
-      <c r="D157" s="5" t="s">
-        <v>559</v>
-      </c>
-      <c r="E157" s="5" t="s">
-        <v>560</v>
       </c>
       <c r="F157" s="5"/>
       <c r="G157" s="5"/>
@@ -6392,19 +6621,19 @@
     </row>
     <row r="158" spans="1:10" ht="42" customHeight="1">
       <c r="A158" s="4" t="s">
+        <v>559</v>
+      </c>
+      <c r="B158" s="7">
+        <v>4</v>
+      </c>
+      <c r="C158" s="8" t="s">
+        <v>658</v>
+      </c>
+      <c r="D158" s="5" t="s">
+        <v>560</v>
+      </c>
+      <c r="E158" s="5" t="s">
         <v>561</v>
-      </c>
-      <c r="B158" s="7">
-        <v>4</v>
-      </c>
-      <c r="C158" s="8" t="s">
-        <v>660</v>
-      </c>
-      <c r="D158" s="5" t="s">
-        <v>562</v>
-      </c>
-      <c r="E158" s="5" t="s">
-        <v>563</v>
       </c>
       <c r="F158" s="5"/>
       <c r="G158" s="5"/>
@@ -6416,19 +6645,19 @@
     </row>
     <row r="159" spans="1:10" ht="42" customHeight="1">
       <c r="A159" s="4" t="s">
-        <v>564</v>
+        <v>562</v>
       </c>
       <c r="B159" s="8">
         <v>6</v>
       </c>
       <c r="C159" s="8" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="D159" s="5" t="s">
-        <v>565</v>
+        <v>563</v>
       </c>
       <c r="E159" s="5" t="s">
-        <v>566</v>
+        <v>564</v>
       </c>
       <c r="F159" s="5"/>
       <c r="G159" s="5"/>
@@ -6440,19 +6669,19 @@
     </row>
     <row r="160" spans="1:10" ht="42" customHeight="1">
       <c r="A160" s="4" t="s">
-        <v>567</v>
+        <v>565</v>
       </c>
       <c r="B160" s="8">
         <v>6</v>
       </c>
       <c r="C160" s="8" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="D160" s="5" t="s">
-        <v>568</v>
+        <v>566</v>
       </c>
       <c r="E160" s="5" t="s">
-        <v>569</v>
+        <v>567</v>
       </c>
       <c r="F160" s="5"/>
       <c r="G160" s="5"/>
@@ -6464,22 +6693,22 @@
     </row>
     <row r="161" spans="1:10" ht="42" customHeight="1">
       <c r="A161" s="4" t="s">
-        <v>570</v>
+        <v>568</v>
       </c>
       <c r="B161" s="8">
         <v>6</v>
       </c>
       <c r="C161" s="8" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="D161" s="5" t="s">
+        <v>569</v>
+      </c>
+      <c r="E161" s="5" t="s">
+        <v>570</v>
+      </c>
+      <c r="F161" s="5" t="s">
         <v>571</v>
-      </c>
-      <c r="E161" s="5" t="s">
-        <v>572</v>
-      </c>
-      <c r="F161" s="5" t="s">
-        <v>573</v>
       </c>
       <c r="G161" s="5"/>
       <c r="H161" s="5"/>
@@ -6490,19 +6719,19 @@
     </row>
     <row r="162" spans="1:10" ht="42" customHeight="1">
       <c r="A162" s="4" t="s">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="B162" s="8">
         <v>6</v>
       </c>
       <c r="C162" s="8" t="s">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="D162" s="5" t="s">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="E162" s="5" t="s">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="F162" s="5"/>
       <c r="G162" s="5"/>
@@ -6514,19 +6743,19 @@
     </row>
     <row r="163" spans="1:10" ht="42" customHeight="1">
       <c r="A163" s="4" t="s">
-        <v>577</v>
+        <v>575</v>
       </c>
       <c r="B163" s="8">
         <v>6</v>
       </c>
       <c r="C163" s="8" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="D163" s="5" t="s">
-        <v>578</v>
+        <v>576</v>
       </c>
       <c r="E163" s="5" t="s">
-        <v>579</v>
+        <v>577</v>
       </c>
       <c r="F163" s="5"/>
       <c r="G163" s="5"/>
@@ -6538,19 +6767,19 @@
     </row>
     <row r="164" spans="1:10" ht="42" customHeight="1">
       <c r="A164" s="4" t="s">
-        <v>580</v>
+        <v>578</v>
       </c>
       <c r="B164" s="8">
         <v>6</v>
       </c>
       <c r="C164" s="8" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="D164" s="5" t="s">
-        <v>581</v>
+        <v>579</v>
       </c>
       <c r="E164" s="5" t="s">
-        <v>582</v>
+        <v>580</v>
       </c>
       <c r="F164" s="5"/>
       <c r="G164" s="5"/>
@@ -6562,19 +6791,19 @@
     </row>
     <row r="165" spans="1:10" ht="42" customHeight="1">
       <c r="A165" s="4" t="s">
-        <v>583</v>
+        <v>581</v>
       </c>
       <c r="B165" s="8">
         <v>6</v>
       </c>
       <c r="C165" s="8" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="D165" s="5" t="s">
-        <v>584</v>
+        <v>582</v>
       </c>
       <c r="E165" s="5" t="s">
-        <v>585</v>
+        <v>583</v>
       </c>
       <c r="F165" s="5"/>
       <c r="G165" s="5"/>
@@ -6586,19 +6815,19 @@
     </row>
     <row r="166" spans="1:10" ht="42" customHeight="1">
       <c r="A166" s="4" t="s">
-        <v>586</v>
+        <v>584</v>
       </c>
       <c r="B166" s="8">
         <v>6</v>
       </c>
       <c r="C166" s="8" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="D166" s="5" t="s">
-        <v>587</v>
+        <v>585</v>
       </c>
       <c r="E166" s="5" t="s">
-        <v>588</v>
+        <v>586</v>
       </c>
       <c r="F166" s="5"/>
       <c r="G166" s="5"/>
@@ -6610,22 +6839,22 @@
     </row>
     <row r="167" spans="1:10" ht="42" customHeight="1">
       <c r="A167" s="4" t="s">
-        <v>589</v>
+        <v>587</v>
       </c>
       <c r="B167" s="8">
         <v>6</v>
       </c>
       <c r="C167" s="8" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="D167" s="5" t="s">
+        <v>588</v>
+      </c>
+      <c r="E167" s="5" t="s">
+        <v>589</v>
+      </c>
+      <c r="F167" s="5" t="s">
         <v>590</v>
-      </c>
-      <c r="E167" s="5" t="s">
-        <v>591</v>
-      </c>
-      <c r="F167" s="5" t="s">
-        <v>592</v>
       </c>
       <c r="G167" s="5"/>
       <c r="H167" s="5"/>
@@ -6636,19 +6865,19 @@
     </row>
     <row r="168" spans="1:10" ht="42" customHeight="1">
       <c r="A168" s="4" t="s">
-        <v>593</v>
+        <v>591</v>
       </c>
       <c r="B168" s="8">
         <v>6</v>
       </c>
       <c r="C168" s="8" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="D168" s="5" t="s">
-        <v>594</v>
+        <v>592</v>
       </c>
       <c r="E168" s="5" t="s">
-        <v>595</v>
+        <v>593</v>
       </c>
       <c r="F168" s="5"/>
       <c r="G168" s="5"/>
@@ -6660,22 +6889,22 @@
     </row>
     <row r="169" spans="1:10" ht="42" customHeight="1">
       <c r="A169" s="4" t="s">
-        <v>596</v>
+        <v>594</v>
       </c>
       <c r="B169" s="8">
         <v>6</v>
       </c>
       <c r="C169" s="8" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="D169" s="5" t="s">
+        <v>595</v>
+      </c>
+      <c r="E169" s="5" t="s">
+        <v>596</v>
+      </c>
+      <c r="F169" s="5" t="s">
         <v>597</v>
-      </c>
-      <c r="E169" s="5" t="s">
-        <v>598</v>
-      </c>
-      <c r="F169" s="5" t="s">
-        <v>599</v>
       </c>
       <c r="G169" s="5"/>
       <c r="H169" s="5"/>
@@ -6686,22 +6915,22 @@
     </row>
     <row r="170" spans="1:10" ht="42" customHeight="1">
       <c r="A170" s="4" t="s">
-        <v>600</v>
+        <v>598</v>
       </c>
       <c r="B170" s="8">
         <v>6</v>
       </c>
       <c r="C170" s="8" t="s">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="D170" s="5" t="s">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="E170" s="5" t="s">
         <v>189</v>
       </c>
       <c r="F170" s="5" t="s">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="G170" s="5"/>
       <c r="H170" s="5"/>
@@ -6712,22 +6941,22 @@
     </row>
     <row r="171" spans="1:10" ht="42" customHeight="1">
       <c r="A171" s="4" t="s">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="B171" s="8">
         <v>6</v>
       </c>
       <c r="C171" s="8" t="s">
-        <v>663</v>
+        <v>661</v>
       </c>
       <c r="D171" s="5" t="s">
+        <v>602</v>
+      </c>
+      <c r="E171" s="5" t="s">
+        <v>603</v>
+      </c>
+      <c r="F171" s="5" t="s">
         <v>604</v>
-      </c>
-      <c r="E171" s="5" t="s">
-        <v>605</v>
-      </c>
-      <c r="F171" s="5" t="s">
-        <v>606</v>
       </c>
       <c r="G171" s="5"/>
       <c r="H171" s="5"/>
@@ -6738,22 +6967,22 @@
     </row>
     <row r="172" spans="1:10" ht="42" customHeight="1">
       <c r="A172" s="4" t="s">
-        <v>607</v>
+        <v>605</v>
       </c>
       <c r="B172" s="8">
         <v>6</v>
       </c>
       <c r="C172" s="8" t="s">
-        <v>663</v>
+        <v>661</v>
       </c>
       <c r="D172" s="5" t="s">
+        <v>606</v>
+      </c>
+      <c r="E172" s="5" t="s">
+        <v>607</v>
+      </c>
+      <c r="F172" s="5" t="s">
         <v>608</v>
-      </c>
-      <c r="E172" s="5" t="s">
-        <v>609</v>
-      </c>
-      <c r="F172" s="5" t="s">
-        <v>610</v>
       </c>
       <c r="G172" s="5"/>
       <c r="H172" s="5"/>
@@ -6764,22 +6993,22 @@
     </row>
     <row r="173" spans="1:10" ht="42" customHeight="1">
       <c r="A173" s="4" t="s">
-        <v>611</v>
+        <v>609</v>
       </c>
       <c r="B173" s="8">
         <v>6</v>
       </c>
       <c r="C173" s="8" t="s">
-        <v>663</v>
+        <v>661</v>
       </c>
       <c r="D173" s="5" t="s">
+        <v>610</v>
+      </c>
+      <c r="E173" s="5" t="s">
+        <v>611</v>
+      </c>
+      <c r="F173" s="5" t="s">
         <v>612</v>
-      </c>
-      <c r="E173" s="5" t="s">
-        <v>613</v>
-      </c>
-      <c r="F173" s="5" t="s">
-        <v>614</v>
       </c>
       <c r="G173" s="5"/>
       <c r="H173" s="5"/>
@@ -6790,22 +7019,22 @@
     </row>
     <row r="174" spans="1:10" ht="42" customHeight="1">
       <c r="A174" s="4" t="s">
-        <v>615</v>
+        <v>613</v>
       </c>
       <c r="B174" s="8">
         <v>6</v>
       </c>
       <c r="C174" s="8" t="s">
-        <v>663</v>
+        <v>661</v>
       </c>
       <c r="D174" s="5" t="s">
+        <v>614</v>
+      </c>
+      <c r="E174" s="5" t="s">
+        <v>615</v>
+      </c>
+      <c r="F174" s="5" t="s">
         <v>616</v>
-      </c>
-      <c r="E174" s="5" t="s">
-        <v>617</v>
-      </c>
-      <c r="F174" s="5" t="s">
-        <v>618</v>
       </c>
       <c r="G174" s="5"/>
       <c r="H174" s="5"/>
@@ -6816,19 +7045,19 @@
     </row>
     <row r="175" spans="1:10" ht="42" customHeight="1">
       <c r="A175" s="4" t="s">
-        <v>619</v>
+        <v>617</v>
       </c>
       <c r="B175" s="8">
         <v>6</v>
       </c>
       <c r="C175" s="8" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
       <c r="D175" s="5" t="s">
-        <v>620</v>
+        <v>618</v>
       </c>
       <c r="E175" s="5" t="s">
-        <v>621</v>
+        <v>619</v>
       </c>
       <c r="F175" s="5"/>
       <c r="G175" s="5"/>
@@ -6840,19 +7069,19 @@
     </row>
     <row r="176" spans="1:10" ht="42" customHeight="1">
       <c r="A176" s="4" t="s">
-        <v>622</v>
+        <v>620</v>
       </c>
       <c r="B176" s="8">
         <v>6</v>
       </c>
       <c r="C176" s="8" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
       <c r="D176" s="5" t="s">
-        <v>623</v>
+        <v>621</v>
       </c>
       <c r="E176" s="5" t="s">
-        <v>624</v>
+        <v>622</v>
       </c>
       <c r="F176" s="5"/>
       <c r="G176" s="5"/>
@@ -6864,19 +7093,19 @@
     </row>
     <row r="177" spans="1:10" ht="42" customHeight="1">
       <c r="A177" s="4" t="s">
-        <v>625</v>
+        <v>623</v>
       </c>
       <c r="B177" s="8">
         <v>6</v>
       </c>
       <c r="C177" s="8" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
       <c r="D177" s="5" t="s">
-        <v>626</v>
+        <v>624</v>
       </c>
       <c r="E177" s="5" t="s">
-        <v>627</v>
+        <v>625</v>
       </c>
       <c r="F177" s="5"/>
       <c r="G177" s="5"/>
@@ -6888,19 +7117,19 @@
     </row>
     <row r="178" spans="1:10" ht="42" customHeight="1">
       <c r="A178" s="4" t="s">
-        <v>628</v>
+        <v>626</v>
       </c>
       <c r="B178" s="8">
         <v>6</v>
       </c>
       <c r="C178" s="8" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
       <c r="D178" s="5" t="s">
-        <v>629</v>
+        <v>627</v>
       </c>
       <c r="E178" s="5" t="s">
-        <v>630</v>
+        <v>628</v>
       </c>
       <c r="F178" s="5"/>
       <c r="G178" s="5"/>
@@ -6912,19 +7141,19 @@
     </row>
     <row r="179" spans="1:10" ht="42" customHeight="1">
       <c r="A179" s="4" t="s">
-        <v>631</v>
+        <v>629</v>
       </c>
       <c r="B179" s="8">
         <v>6</v>
       </c>
       <c r="C179" s="8" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
       <c r="D179" s="5" t="s">
-        <v>632</v>
+        <v>630</v>
       </c>
       <c r="E179" s="5" t="s">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="F179" s="5"/>
       <c r="G179" s="5"/>
@@ -6936,19 +7165,19 @@
     </row>
     <row r="180" spans="1:10" ht="42" customHeight="1">
       <c r="A180" s="4" t="s">
-        <v>634</v>
+        <v>632</v>
       </c>
       <c r="B180" s="8">
         <v>6</v>
       </c>
       <c r="C180" s="8" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
       <c r="D180" s="5" t="s">
-        <v>635</v>
+        <v>633</v>
       </c>
       <c r="E180" s="5" t="s">
-        <v>636</v>
+        <v>634</v>
       </c>
       <c r="F180" s="5"/>
       <c r="G180" s="5"/>
@@ -6960,19 +7189,19 @@
     </row>
     <row r="181" spans="1:10" ht="42" customHeight="1">
       <c r="A181" s="4" t="s">
-        <v>637</v>
+        <v>635</v>
       </c>
       <c r="B181" s="8">
         <v>6</v>
       </c>
       <c r="C181" s="8" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
       <c r="D181" s="5" t="s">
-        <v>638</v>
+        <v>636</v>
       </c>
       <c r="E181" s="5" t="s">
-        <v>639</v>
+        <v>637</v>
       </c>
       <c r="F181" s="5"/>
       <c r="G181" s="5"/>
@@ -6984,22 +7213,22 @@
     </row>
     <row r="182" spans="1:10" ht="42" customHeight="1">
       <c r="A182" s="4" t="s">
-        <v>640</v>
+        <v>638</v>
       </c>
       <c r="B182" s="8">
         <v>6</v>
       </c>
       <c r="C182" s="8" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
       <c r="D182" s="5" t="s">
+        <v>639</v>
+      </c>
+      <c r="E182" s="5" t="s">
+        <v>640</v>
+      </c>
+      <c r="F182" s="5" t="s">
         <v>641</v>
-      </c>
-      <c r="E182" s="5" t="s">
-        <v>642</v>
-      </c>
-      <c r="F182" s="5" t="s">
-        <v>643</v>
       </c>
       <c r="G182" s="5"/>
       <c r="H182" s="5"/>
@@ -7010,19 +7239,19 @@
     </row>
     <row r="183" spans="1:10" ht="42" customHeight="1">
       <c r="A183" s="4" t="s">
-        <v>644</v>
+        <v>642</v>
       </c>
       <c r="B183" s="8">
         <v>6</v>
       </c>
       <c r="C183" s="8" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
       <c r="D183" s="5" t="s">
-        <v>645</v>
+        <v>643</v>
       </c>
       <c r="E183" s="5" t="s">
-        <v>646</v>
+        <v>644</v>
       </c>
       <c r="F183" s="5"/>
       <c r="G183" s="5"/>
@@ -7034,19 +7263,19 @@
     </row>
     <row r="184" spans="1:10" ht="42" customHeight="1">
       <c r="A184" s="4" t="s">
-        <v>647</v>
+        <v>645</v>
       </c>
       <c r="B184" s="8">
         <v>6</v>
       </c>
       <c r="C184" s="8" t="s">
-        <v>664</v>
+        <v>662</v>
       </c>
       <c r="D184" s="5" t="s">
-        <v>648</v>
+        <v>646</v>
       </c>
       <c r="E184" s="5" t="s">
-        <v>649</v>
+        <v>647</v>
       </c>
       <c r="F184" s="5"/>
       <c r="G184" s="5"/>
@@ -7056,10 +7285,322 @@
         <v>14</v>
       </c>
     </row>
+    <row r="185" spans="1:10" ht="42" customHeight="1">
+      <c r="A185" s="4" t="s">
+        <v>665</v>
+      </c>
+      <c r="B185" s="8">
+        <v>6</v>
+      </c>
+      <c r="C185" s="8" t="s">
+        <v>680</v>
+      </c>
+      <c r="D185" s="5" t="s">
+        <v>681</v>
+      </c>
+      <c r="E185" s="5" t="s">
+        <v>699</v>
+      </c>
+      <c r="F185" s="5"/>
+    </row>
+    <row r="186" spans="1:10" ht="42" customHeight="1">
+      <c r="A186" s="4" t="s">
+        <v>666</v>
+      </c>
+      <c r="B186" s="8">
+        <v>6</v>
+      </c>
+      <c r="C186" s="8" t="s">
+        <v>680</v>
+      </c>
+      <c r="D186" s="5" t="s">
+        <v>682</v>
+      </c>
+      <c r="E186" s="5" t="s">
+        <v>700</v>
+      </c>
+      <c r="F186" s="5" t="s">
+        <v>715</v>
+      </c>
+    </row>
+    <row r="187" spans="1:10" ht="42" customHeight="1">
+      <c r="A187" s="4" t="s">
+        <v>667</v>
+      </c>
+      <c r="B187" s="8">
+        <v>6</v>
+      </c>
+      <c r="C187" s="8" t="s">
+        <v>680</v>
+      </c>
+      <c r="D187" s="5" t="s">
+        <v>683</v>
+      </c>
+      <c r="E187" s="5" t="s">
+        <v>701</v>
+      </c>
+      <c r="F187" s="5" t="s">
+        <v>716</v>
+      </c>
+    </row>
+    <row r="188" spans="1:10" ht="42" customHeight="1">
+      <c r="A188" s="4" t="s">
+        <v>668</v>
+      </c>
+      <c r="B188" s="8">
+        <v>6</v>
+      </c>
+      <c r="C188" s="8" t="s">
+        <v>679</v>
+      </c>
+      <c r="D188" s="5" t="s">
+        <v>684</v>
+      </c>
+      <c r="E188" s="5" t="s">
+        <v>702</v>
+      </c>
+      <c r="F188" s="5" t="s">
+        <v>717</v>
+      </c>
+    </row>
+    <row r="189" spans="1:10" ht="42" customHeight="1">
+      <c r="A189" s="4" t="s">
+        <v>669</v>
+      </c>
+      <c r="B189" s="8">
+        <v>6</v>
+      </c>
+      <c r="C189" s="8" t="s">
+        <v>679</v>
+      </c>
+      <c r="D189" s="5" t="s">
+        <v>685</v>
+      </c>
+      <c r="E189" s="5" t="s">
+        <v>703</v>
+      </c>
+      <c r="F189" s="5"/>
+    </row>
+    <row r="190" spans="1:10" ht="42" customHeight="1">
+      <c r="A190" s="4" t="s">
+        <v>670</v>
+      </c>
+      <c r="B190" s="8">
+        <v>6</v>
+      </c>
+      <c r="C190" s="8" t="s">
+        <v>679</v>
+      </c>
+      <c r="D190" s="5" t="s">
+        <v>686</v>
+      </c>
+      <c r="E190" s="5" t="s">
+        <v>704</v>
+      </c>
+      <c r="F190" s="5"/>
+    </row>
+    <row r="191" spans="1:10" ht="42" customHeight="1">
+      <c r="A191" s="4" t="s">
+        <v>671</v>
+      </c>
+      <c r="B191" s="8">
+        <v>6</v>
+      </c>
+      <c r="C191" s="8" t="s">
+        <v>679</v>
+      </c>
+      <c r="D191" s="5" t="s">
+        <v>687</v>
+      </c>
+      <c r="E191" s="5" t="s">
+        <v>705</v>
+      </c>
+      <c r="F191" s="5" t="s">
+        <v>718</v>
+      </c>
+    </row>
+    <row r="192" spans="1:10" ht="42" customHeight="1">
+      <c r="A192" s="4" t="s">
+        <v>672</v>
+      </c>
+      <c r="B192" s="8">
+        <v>6</v>
+      </c>
+      <c r="C192" s="8" t="s">
+        <v>679</v>
+      </c>
+      <c r="D192" s="5" t="s">
+        <v>688</v>
+      </c>
+      <c r="E192" s="5" t="s">
+        <v>706</v>
+      </c>
+      <c r="F192" s="5" t="s">
+        <v>719</v>
+      </c>
+    </row>
+    <row r="193" spans="1:6" ht="42" customHeight="1">
+      <c r="A193" s="4" t="s">
+        <v>673</v>
+      </c>
+      <c r="B193" s="8">
+        <v>6</v>
+      </c>
+      <c r="C193" s="8" t="s">
+        <v>679</v>
+      </c>
+      <c r="D193" s="5" t="s">
+        <v>689</v>
+      </c>
+      <c r="E193" s="5" t="s">
+        <v>707</v>
+      </c>
+      <c r="F193" s="5" t="s">
+        <v>720</v>
+      </c>
+    </row>
+    <row r="194" spans="1:6" ht="42" customHeight="1">
+      <c r="A194" s="4" t="s">
+        <v>674</v>
+      </c>
+      <c r="B194" s="8">
+        <v>6</v>
+      </c>
+      <c r="C194" s="8" t="s">
+        <v>679</v>
+      </c>
+      <c r="D194" s="5" t="s">
+        <v>690</v>
+      </c>
+      <c r="E194" s="5" t="s">
+        <v>708</v>
+      </c>
+      <c r="F194" s="5"/>
+    </row>
+    <row r="195" spans="1:6" ht="42" customHeight="1">
+      <c r="A195" s="4" t="s">
+        <v>675</v>
+      </c>
+      <c r="B195" s="8">
+        <v>6</v>
+      </c>
+      <c r="C195" s="8" t="s">
+        <v>679</v>
+      </c>
+      <c r="D195" s="5" t="s">
+        <v>691</v>
+      </c>
+      <c r="E195" s="5" t="s">
+        <v>709</v>
+      </c>
+      <c r="F195" s="5" t="s">
+        <v>721</v>
+      </c>
+    </row>
+    <row r="196" spans="1:6" ht="42" customHeight="1">
+      <c r="A196" s="4" t="s">
+        <v>676</v>
+      </c>
+      <c r="B196" s="8">
+        <v>6</v>
+      </c>
+      <c r="C196" s="8" t="s">
+        <v>679</v>
+      </c>
+      <c r="D196" s="5" t="s">
+        <v>692</v>
+      </c>
+      <c r="E196" s="5" t="s">
+        <v>710</v>
+      </c>
+      <c r="F196" s="5" t="s">
+        <v>722</v>
+      </c>
+    </row>
+    <row r="197" spans="1:6" ht="42" customHeight="1">
+      <c r="A197" s="4" t="s">
+        <v>677</v>
+      </c>
+      <c r="B197" s="8">
+        <v>6</v>
+      </c>
+      <c r="C197" s="8" t="s">
+        <v>679</v>
+      </c>
+      <c r="D197" s="5" t="s">
+        <v>693</v>
+      </c>
+      <c r="E197" s="5" t="s">
+        <v>711</v>
+      </c>
+      <c r="F197" s="5" t="s">
+        <v>723</v>
+      </c>
+    </row>
+    <row r="198" spans="1:6" ht="42" customHeight="1">
+      <c r="A198" s="4" t="s">
+        <v>678</v>
+      </c>
+      <c r="B198" s="8">
+        <v>6</v>
+      </c>
+      <c r="C198" s="8" t="s">
+        <v>679</v>
+      </c>
+      <c r="D198" s="5" t="s">
+        <v>694</v>
+      </c>
+      <c r="E198" s="5" t="s">
+        <v>712</v>
+      </c>
+      <c r="F198" s="5" t="s">
+        <v>724</v>
+      </c>
+    </row>
+    <row r="199" spans="1:6" ht="42" customHeight="1">
+      <c r="A199" s="4" t="s">
+        <v>695</v>
+      </c>
+      <c r="B199" s="8">
+        <v>6</v>
+      </c>
+      <c r="C199" s="8" t="s">
+        <v>679</v>
+      </c>
+      <c r="D199" s="5" t="s">
+        <v>697</v>
+      </c>
+      <c r="E199" s="5" t="s">
+        <v>713</v>
+      </c>
+      <c r="F199" s="5" t="s">
+        <v>724</v>
+      </c>
+    </row>
+    <row r="200" spans="1:6" ht="42" customHeight="1">
+      <c r="A200" s="4" t="s">
+        <v>696</v>
+      </c>
+      <c r="B200" s="8">
+        <v>6</v>
+      </c>
+      <c r="C200" s="8" t="s">
+        <v>679</v>
+      </c>
+      <c r="D200" s="5" t="s">
+        <v>698</v>
+      </c>
+      <c r="E200" s="5" t="s">
+        <v>714</v>
+      </c>
+      <c r="F200" s="5" t="s">
+        <v>725</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="4" type="noConversion"/>
   <conditionalFormatting sqref="I2:I158">
-    <cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="yes"/>
+    <cfRule type="containsText" dxfId="2" priority="1" operator="containsText" text="yes"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">

</xml_diff>

<commit_message>
Preserve scientific rich text formatting
</commit_message>
<xml_diff>
--- a/data/question-bank.xlsx
+++ b/data/question-bank.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/adamsun/Documents/Codex/exam-recall-trainer/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9900D2CD-37B6-F742-AD4D-432D0CD721C1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FCE988A4-F3A6-F34C-B36F-568EDC55939E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="920" yWindow="600" windowWidth="27140" windowHeight="15100" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4220,10 +4220,6 @@
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
   <si>
-    <t>As [A−] : [HA] ratio is unchanged</t>
-    <phoneticPr fontId="4" type="noConversion"/>
-  </si>
-  <si>
     <t>Describe the difference between an element and a compound</t>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
@@ -5520,6 +5516,27 @@
   </si>
   <si>
     <t>More soluble impurity removed: removing / filtering crystals from cold solution</t>
+    <phoneticPr fontId="4" type="noConversion"/>
+  </si>
+  <si>
+    <r>
+      <t>As [A</t>
+    </r>
+    <r>
+      <rPr>
+        <vertAlign val="superscript"/>
+        <sz val="11"/>
+        <rFont val="Aptos"/>
+      </rPr>
+      <t>−</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Aptos"/>
+      </rPr>
+      <t>] : [HA] ratio is unchanged</t>
+    </r>
     <phoneticPr fontId="4" type="noConversion"/>
   </si>
 </sst>
@@ -11730,7 +11747,7 @@
     </row>
     <row r="2" spans="1:10" ht="42" customHeight="1">
       <c r="A2" s="2" t="s">
-        <v>996</v>
+        <v>995</v>
       </c>
       <c r="B2" s="7">
         <v>2</v>
@@ -11739,13 +11756,13 @@
         <v>833</v>
       </c>
       <c r="D2" s="3" t="s">
+        <v>898</v>
+      </c>
+      <c r="E2" s="3" t="s">
         <v>899</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="F2" s="3" t="s">
         <v>900</v>
-      </c>
-      <c r="F2" s="3" t="s">
-        <v>901</v>
       </c>
       <c r="G2" s="3"/>
       <c r="H2" s="3"/>
@@ -11754,7 +11771,7 @@
     </row>
     <row r="3" spans="1:10" ht="42" customHeight="1">
       <c r="A3" s="2" t="s">
-        <v>997</v>
+        <v>996</v>
       </c>
       <c r="B3" s="7">
         <v>2</v>
@@ -11763,13 +11780,13 @@
         <v>833</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>963</v>
+        <v>962</v>
       </c>
       <c r="E3" s="3" t="s">
+        <v>967</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>968</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>969</v>
       </c>
       <c r="G3" s="3"/>
       <c r="H3" s="3"/>
@@ -11778,7 +11795,7 @@
     </row>
     <row r="4" spans="1:10" ht="42" customHeight="1">
       <c r="A4" s="2" t="s">
-        <v>998</v>
+        <v>997</v>
       </c>
       <c r="B4" s="7">
         <v>2</v>
@@ -11787,13 +11804,13 @@
         <v>833</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>964</v>
+        <v>963</v>
       </c>
       <c r="E4" s="3" t="s">
+        <v>965</v>
+      </c>
+      <c r="F4" s="3" t="s">
         <v>966</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>967</v>
       </c>
       <c r="G4" s="3"/>
       <c r="H4" s="3"/>
@@ -11802,7 +11819,7 @@
     </row>
     <row r="5" spans="1:10" ht="42" customHeight="1">
       <c r="A5" s="2" t="s">
-        <v>999</v>
+        <v>998</v>
       </c>
       <c r="B5" s="7">
         <v>2</v>
@@ -11811,13 +11828,13 @@
         <v>833</v>
       </c>
       <c r="D5" s="12" t="s">
+        <v>964</v>
+      </c>
+      <c r="E5" s="3" t="s">
         <v>965</v>
       </c>
-      <c r="E5" s="3" t="s">
-        <v>966</v>
-      </c>
       <c r="F5" s="3" t="s">
-        <v>970</v>
+        <v>969</v>
       </c>
       <c r="G5" s="3"/>
       <c r="H5" s="3"/>
@@ -11826,7 +11843,7 @@
     </row>
     <row r="6" spans="1:10" ht="42" customHeight="1">
       <c r="A6" s="2" t="s">
-        <v>1000</v>
+        <v>999</v>
       </c>
       <c r="B6" s="8">
         <v>2</v>
@@ -11835,10 +11852,10 @@
         <v>833</v>
       </c>
       <c r="D6" s="5" t="s">
+        <v>939</v>
+      </c>
+      <c r="E6" s="5" t="s">
         <v>940</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>941</v>
       </c>
       <c r="F6" s="5"/>
       <c r="G6" s="5"/>
@@ -11848,7 +11865,7 @@
     </row>
     <row r="7" spans="1:10" ht="42" customHeight="1">
       <c r="A7" s="2" t="s">
-        <v>1001</v>
+        <v>1000</v>
       </c>
       <c r="B7" s="8">
         <v>2</v>
@@ -11857,10 +11874,10 @@
         <v>834</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>910</v>
+        <v>909</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>912</v>
+        <v>911</v>
       </c>
       <c r="F7" s="5"/>
       <c r="G7" s="5"/>
@@ -11870,7 +11887,7 @@
     </row>
     <row r="8" spans="1:10" ht="42" customHeight="1">
       <c r="A8" s="2" t="s">
-        <v>1002</v>
+        <v>1001</v>
       </c>
       <c r="B8" s="8">
         <v>2</v>
@@ -11879,10 +11896,10 @@
         <v>834</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>911</v>
+        <v>910</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>913</v>
+        <v>912</v>
       </c>
       <c r="F8" s="5"/>
       <c r="G8" s="5"/>
@@ -11892,7 +11909,7 @@
     </row>
     <row r="9" spans="1:10" ht="42" customHeight="1">
       <c r="A9" s="2" t="s">
-        <v>1003</v>
+        <v>1002</v>
       </c>
       <c r="B9" s="8">
         <v>2</v>
@@ -11901,13 +11918,13 @@
         <v>834</v>
       </c>
       <c r="D9" s="5" t="s">
+        <v>934</v>
+      </c>
+      <c r="E9" s="5" t="s">
         <v>935</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="F9" s="5" t="s">
         <v>936</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>937</v>
       </c>
       <c r="G9" s="5"/>
       <c r="H9" s="5"/>
@@ -11916,7 +11933,7 @@
     </row>
     <row r="10" spans="1:10" ht="42" customHeight="1">
       <c r="A10" s="2" t="s">
-        <v>1004</v>
+        <v>1003</v>
       </c>
       <c r="B10" s="8">
         <v>2</v>
@@ -11925,10 +11942,10 @@
         <v>834</v>
       </c>
       <c r="D10" s="5" t="s">
+        <v>937</v>
+      </c>
+      <c r="E10" s="5" t="s">
         <v>938</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>939</v>
       </c>
       <c r="F10" s="5"/>
       <c r="G10" s="5"/>
@@ -11938,7 +11955,7 @@
     </row>
     <row r="11" spans="1:10" ht="42" customHeight="1">
       <c r="A11" s="2" t="s">
-        <v>1005</v>
+        <v>1004</v>
       </c>
       <c r="B11" s="8">
         <v>2</v>
@@ -11947,13 +11964,13 @@
         <v>834</v>
       </c>
       <c r="D11" s="5" t="s">
+        <v>923</v>
+      </c>
+      <c r="E11" s="5" t="s">
         <v>924</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="F11" s="5" t="s">
         <v>925</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>926</v>
       </c>
       <c r="G11" s="5"/>
       <c r="H11" s="5"/>
@@ -11962,7 +11979,7 @@
     </row>
     <row r="12" spans="1:10" ht="42" customHeight="1">
       <c r="A12" s="2" t="s">
-        <v>1006</v>
+        <v>1005</v>
       </c>
       <c r="B12" s="8">
         <v>2</v>
@@ -11984,7 +12001,7 @@
     </row>
     <row r="13" spans="1:10" ht="42" customHeight="1">
       <c r="A13" s="2" t="s">
-        <v>1007</v>
+        <v>1006</v>
       </c>
       <c r="B13" s="8">
         <v>2</v>
@@ -12006,7 +12023,7 @@
     </row>
     <row r="14" spans="1:10" ht="42" customHeight="1">
       <c r="A14" s="2" t="s">
-        <v>1008</v>
+        <v>1007</v>
       </c>
       <c r="B14" s="8">
         <v>2</v>
@@ -12030,7 +12047,7 @@
     </row>
     <row r="15" spans="1:10" ht="42" customHeight="1">
       <c r="A15" s="2" t="s">
-        <v>1009</v>
+        <v>1008</v>
       </c>
       <c r="B15" s="8">
         <v>2</v>
@@ -12052,7 +12069,7 @@
     </row>
     <row r="16" spans="1:10" ht="42" customHeight="1">
       <c r="A16" s="2" t="s">
-        <v>1010</v>
+        <v>1009</v>
       </c>
       <c r="B16" s="8">
         <v>2</v>
@@ -12076,7 +12093,7 @@
     </row>
     <row r="17" spans="1:10" ht="42" customHeight="1">
       <c r="A17" s="2" t="s">
-        <v>1011</v>
+        <v>1010</v>
       </c>
       <c r="B17" s="8">
         <v>2</v>
@@ -12102,7 +12119,7 @@
     </row>
     <row r="18" spans="1:10" ht="42" customHeight="1">
       <c r="A18" s="2" t="s">
-        <v>1012</v>
+        <v>1011</v>
       </c>
       <c r="B18" s="8">
         <v>2</v>
@@ -12111,13 +12128,13 @@
         <v>834</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>920</v>
+        <v>919</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>993</v>
+        <v>992</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>919</v>
+        <v>918</v>
       </c>
       <c r="G18" s="11"/>
       <c r="H18" s="5"/>
@@ -12126,7 +12143,7 @@
     </row>
     <row r="19" spans="1:10" ht="42" customHeight="1">
       <c r="A19" s="2" t="s">
-        <v>1013</v>
+        <v>1012</v>
       </c>
       <c r="B19" s="8">
         <v>2</v>
@@ -12135,10 +12152,10 @@
         <v>834</v>
       </c>
       <c r="D19" s="5" t="s">
+        <v>920</v>
+      </c>
+      <c r="E19" s="5" t="s">
         <v>921</v>
-      </c>
-      <c r="E19" s="5" t="s">
-        <v>922</v>
       </c>
       <c r="F19" s="5"/>
       <c r="G19" s="11"/>
@@ -12148,7 +12165,7 @@
     </row>
     <row r="20" spans="1:10" ht="42" customHeight="1">
       <c r="A20" s="2" t="s">
-        <v>1014</v>
+        <v>1013</v>
       </c>
       <c r="B20" s="8">
         <v>2</v>
@@ -12157,13 +12174,13 @@
         <v>834</v>
       </c>
       <c r="D20" s="5" t="s">
+        <v>983</v>
+      </c>
+      <c r="E20" s="5" t="s">
         <v>984</v>
       </c>
-      <c r="E20" s="5" t="s">
+      <c r="F20" s="5" t="s">
         <v>985</v>
-      </c>
-      <c r="F20" s="5" t="s">
-        <v>986</v>
       </c>
       <c r="G20" s="11"/>
       <c r="H20" s="5"/>
@@ -12172,7 +12189,7 @@
     </row>
     <row r="21" spans="1:10" ht="42" customHeight="1">
       <c r="A21" s="2" t="s">
-        <v>1015</v>
+        <v>1014</v>
       </c>
       <c r="B21" s="8">
         <v>2</v>
@@ -12196,7 +12213,7 @@
     </row>
     <row r="22" spans="1:10" ht="42" customHeight="1">
       <c r="A22" s="2" t="s">
-        <v>1016</v>
+        <v>1015</v>
       </c>
       <c r="B22" s="8">
         <v>2</v>
@@ -12205,10 +12222,10 @@
         <v>834</v>
       </c>
       <c r="D22" s="5" t="s">
+        <v>913</v>
+      </c>
+      <c r="E22" s="5" t="s">
         <v>914</v>
-      </c>
-      <c r="E22" s="5" t="s">
-        <v>915</v>
       </c>
       <c r="F22" s="5"/>
       <c r="G22" s="11"/>
@@ -12218,7 +12235,7 @@
     </row>
     <row r="23" spans="1:10" ht="42" customHeight="1">
       <c r="A23" s="2" t="s">
-        <v>1017</v>
+        <v>1016</v>
       </c>
       <c r="B23" s="7">
         <v>2</v>
@@ -12241,7 +12258,7 @@
     </row>
     <row r="24" spans="1:10" ht="42" customHeight="1">
       <c r="A24" s="2" t="s">
-        <v>1018</v>
+        <v>1017</v>
       </c>
       <c r="B24" s="7">
         <v>2</v>
@@ -12250,13 +12267,13 @@
         <v>835</v>
       </c>
       <c r="D24" s="5" t="s">
+        <v>941</v>
+      </c>
+      <c r="E24" s="5" t="s">
         <v>942</v>
       </c>
-      <c r="E24" s="5" t="s">
+      <c r="F24" s="5" t="s">
         <v>943</v>
-      </c>
-      <c r="F24" s="5" t="s">
-        <v>944</v>
       </c>
       <c r="H24" s="5"/>
       <c r="I24" s="5"/>
@@ -12264,7 +12281,7 @@
     </row>
     <row r="25" spans="1:10" ht="42" customHeight="1">
       <c r="A25" s="2" t="s">
-        <v>1019</v>
+        <v>1018</v>
       </c>
       <c r="B25" s="8">
         <v>2</v>
@@ -12288,7 +12305,7 @@
     </row>
     <row r="26" spans="1:10" ht="42" customHeight="1">
       <c r="A26" s="2" t="s">
-        <v>1020</v>
+        <v>1019</v>
       </c>
       <c r="B26" s="8">
         <v>2</v>
@@ -12314,7 +12331,7 @@
     </row>
     <row r="27" spans="1:10" ht="42" customHeight="1">
       <c r="A27" s="2" t="s">
-        <v>1021</v>
+        <v>1020</v>
       </c>
       <c r="B27" s="8">
         <v>2</v>
@@ -12323,26 +12340,26 @@
         <v>835</v>
       </c>
       <c r="D27" s="5" t="s">
+        <v>904</v>
+      </c>
+      <c r="E27" s="5" t="s">
         <v>905</v>
       </c>
-      <c r="E27" s="5" t="s">
+      <c r="F27" s="5" t="s">
         <v>906</v>
       </c>
-      <c r="F27" s="5" t="s">
+      <c r="G27" s="5" t="s">
         <v>907</v>
       </c>
-      <c r="G27" s="5" t="s">
+      <c r="H27" s="5" t="s">
         <v>908</v>
-      </c>
-      <c r="H27" s="5" t="s">
-        <v>909</v>
       </c>
       <c r="I27" s="5"/>
       <c r="J27" s="5"/>
     </row>
     <row r="28" spans="1:10" ht="42" customHeight="1">
       <c r="A28" s="2" t="s">
-        <v>1022</v>
+        <v>1021</v>
       </c>
       <c r="B28" s="8">
         <v>2</v>
@@ -12351,13 +12368,13 @@
         <v>835</v>
       </c>
       <c r="D28" s="5" t="s">
+        <v>915</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>917</v>
+      </c>
+      <c r="F28" s="5" t="s">
         <v>916</v>
-      </c>
-      <c r="E28" s="5" t="s">
-        <v>918</v>
-      </c>
-      <c r="F28" s="5" t="s">
-        <v>917</v>
       </c>
       <c r="G28" s="5"/>
       <c r="H28" s="5"/>
@@ -12366,7 +12383,7 @@
     </row>
     <row r="29" spans="1:10" ht="42" customHeight="1">
       <c r="A29" s="2" t="s">
-        <v>1023</v>
+        <v>1022</v>
       </c>
       <c r="B29" s="8">
         <v>2</v>
@@ -12375,10 +12392,10 @@
         <v>835</v>
       </c>
       <c r="D29" s="5" t="s">
+        <v>956</v>
+      </c>
+      <c r="E29" s="5" t="s">
         <v>957</v>
-      </c>
-      <c r="E29" s="5" t="s">
-        <v>958</v>
       </c>
       <c r="F29" s="5"/>
       <c r="G29" s="5"/>
@@ -12388,7 +12405,7 @@
     </row>
     <row r="30" spans="1:10" ht="42" customHeight="1">
       <c r="A30" s="2" t="s">
-        <v>1024</v>
+        <v>1023</v>
       </c>
       <c r="B30" s="8">
         <v>2</v>
@@ -12397,10 +12414,10 @@
         <v>835</v>
       </c>
       <c r="D30" s="5" t="s">
+        <v>954</v>
+      </c>
+      <c r="E30" s="5" t="s">
         <v>955</v>
-      </c>
-      <c r="E30" s="5" t="s">
-        <v>956</v>
       </c>
       <c r="F30" s="5"/>
       <c r="G30" s="5"/>
@@ -12410,16 +12427,16 @@
     </row>
     <row r="31" spans="1:10" ht="42" customHeight="1">
       <c r="A31" s="2" t="s">
-        <v>1025</v>
+        <v>1024</v>
       </c>
       <c r="B31" s="8">
         <v>2</v>
       </c>
       <c r="C31" s="7" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
       <c r="D31" s="5" t="s">
-        <v>923</v>
+        <v>922</v>
       </c>
       <c r="E31" s="5" t="s">
         <v>859</v>
@@ -12434,41 +12451,41 @@
     </row>
     <row r="32" spans="1:10" ht="42" customHeight="1">
       <c r="A32" s="2" t="s">
-        <v>1026</v>
+        <v>1025</v>
       </c>
       <c r="B32" s="8">
         <v>2</v>
       </c>
       <c r="C32" s="7" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
       <c r="D32" s="5" t="s">
+        <v>987</v>
+      </c>
+      <c r="E32" s="5" t="s">
         <v>988</v>
       </c>
-      <c r="E32" s="5" t="s">
+      <c r="F32" s="5" t="s">
         <v>989</v>
       </c>
-      <c r="F32" s="5" t="s">
+      <c r="G32" s="5" t="s">
         <v>990</v>
       </c>
-      <c r="G32" s="5" t="s">
+      <c r="H32" s="5" t="s">
         <v>991</v>
-      </c>
-      <c r="H32" s="5" t="s">
-        <v>992</v>
       </c>
       <c r="I32" s="5"/>
       <c r="J32" s="5"/>
     </row>
     <row r="33" spans="1:10" ht="42" customHeight="1">
       <c r="A33" s="2" t="s">
-        <v>1027</v>
+        <v>1026</v>
       </c>
       <c r="B33" s="8">
         <v>2</v>
       </c>
       <c r="C33" s="7" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
       <c r="D33" s="5" t="s">
         <v>888</v>
@@ -12484,13 +12501,13 @@
     </row>
     <row r="34" spans="1:10" ht="42" customHeight="1">
       <c r="A34" s="2" t="s">
-        <v>1028</v>
+        <v>1027</v>
       </c>
       <c r="B34" s="8">
         <v>2</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>1187</v>
+        <v>1186</v>
       </c>
       <c r="D34" s="5" t="s">
         <v>861</v>
@@ -12510,7 +12527,7 @@
     </row>
     <row r="35" spans="1:10" ht="42" customHeight="1">
       <c r="A35" s="2" t="s">
-        <v>1029</v>
+        <v>1028</v>
       </c>
       <c r="B35" s="7">
         <v>2</v>
@@ -12519,13 +12536,13 @@
         <v>836</v>
       </c>
       <c r="D35" s="5" t="s">
+        <v>944</v>
+      </c>
+      <c r="E35" s="5" t="s">
         <v>945</v>
       </c>
-      <c r="E35" s="5" t="s">
+      <c r="F35" s="5" t="s">
         <v>946</v>
-      </c>
-      <c r="F35" s="5" t="s">
-        <v>947</v>
       </c>
       <c r="G35" s="5"/>
       <c r="H35" s="5"/>
@@ -12534,7 +12551,7 @@
     </row>
     <row r="36" spans="1:10" ht="42" customHeight="1">
       <c r="A36" s="2" t="s">
-        <v>1030</v>
+        <v>1029</v>
       </c>
       <c r="B36" s="7">
         <v>2</v>
@@ -12543,13 +12560,13 @@
         <v>836</v>
       </c>
       <c r="D36" s="5" t="s">
+        <v>951</v>
+      </c>
+      <c r="E36" s="5" t="s">
         <v>952</v>
       </c>
-      <c r="E36" s="5" t="s">
+      <c r="F36" s="5" t="s">
         <v>953</v>
-      </c>
-      <c r="F36" s="5" t="s">
-        <v>954</v>
       </c>
       <c r="G36" s="5"/>
       <c r="H36" s="5"/>
@@ -12558,7 +12575,7 @@
     </row>
     <row r="37" spans="1:10" ht="42" customHeight="1">
       <c r="A37" s="2" t="s">
-        <v>1031</v>
+        <v>1030</v>
       </c>
       <c r="B37" s="7">
         <v>2</v>
@@ -12584,7 +12601,7 @@
     </row>
     <row r="38" spans="1:10" ht="42" customHeight="1">
       <c r="A38" s="2" t="s">
-        <v>1032</v>
+        <v>1031</v>
       </c>
       <c r="B38" s="7">
         <v>2</v>
@@ -12593,26 +12610,26 @@
         <v>836</v>
       </c>
       <c r="D38" s="5" t="s">
+        <v>947</v>
+      </c>
+      <c r="E38" s="5" t="s">
         <v>948</v>
       </c>
-      <c r="E38" s="5" t="s">
+      <c r="F38" s="5" t="s">
         <v>949</v>
       </c>
-      <c r="F38" s="5" t="s">
+      <c r="G38" s="5" t="s">
         <v>950</v>
       </c>
-      <c r="G38" s="5" t="s">
-        <v>951</v>
-      </c>
       <c r="H38" s="5" t="s">
-        <v>987</v>
+        <v>986</v>
       </c>
       <c r="I38" s="5"/>
       <c r="J38" s="5"/>
     </row>
     <row r="39" spans="1:10" ht="42" customHeight="1">
       <c r="A39" s="2" t="s">
-        <v>1033</v>
+        <v>1032</v>
       </c>
       <c r="B39" s="8">
         <v>2</v>
@@ -12636,7 +12653,7 @@
     </row>
     <row r="40" spans="1:10" ht="42" customHeight="1">
       <c r="A40" s="2" t="s">
-        <v>1034</v>
+        <v>1033</v>
       </c>
       <c r="B40" s="8">
         <v>2</v>
@@ -12658,7 +12675,7 @@
     </row>
     <row r="41" spans="1:10" ht="42" customHeight="1">
       <c r="A41" s="2" t="s">
-        <v>1035</v>
+        <v>1034</v>
       </c>
       <c r="B41" s="8">
         <v>2</v>
@@ -12682,7 +12699,7 @@
     </row>
     <row r="42" spans="1:10" ht="42" customHeight="1">
       <c r="A42" s="2" t="s">
-        <v>1036</v>
+        <v>1035</v>
       </c>
       <c r="B42" s="8">
         <v>2</v>
@@ -12691,16 +12708,16 @@
         <v>837</v>
       </c>
       <c r="D42" s="5" t="s">
+        <v>926</v>
+      </c>
+      <c r="E42" s="5" t="s">
         <v>927</v>
       </c>
-      <c r="E42" s="5" t="s">
+      <c r="F42" s="5" t="s">
         <v>928</v>
       </c>
-      <c r="F42" s="5" t="s">
+      <c r="G42" s="5" t="s">
         <v>929</v>
-      </c>
-      <c r="G42" s="5" t="s">
-        <v>930</v>
       </c>
       <c r="H42" s="5"/>
       <c r="I42" s="5"/>
@@ -12708,7 +12725,7 @@
     </row>
     <row r="43" spans="1:10" ht="42" customHeight="1">
       <c r="A43" s="2" t="s">
-        <v>1037</v>
+        <v>1036</v>
       </c>
       <c r="B43" s="8">
         <v>2</v>
@@ -12732,7 +12749,7 @@
     </row>
     <row r="44" spans="1:10" ht="42" customHeight="1">
       <c r="A44" s="2" t="s">
-        <v>1038</v>
+        <v>1037</v>
       </c>
       <c r="B44" s="8">
         <v>2</v>
@@ -12756,7 +12773,7 @@
     </row>
     <row r="45" spans="1:10" ht="42" customHeight="1">
       <c r="A45" s="2" t="s">
-        <v>1039</v>
+        <v>1038</v>
       </c>
       <c r="B45" s="8">
         <v>2</v>
@@ -12765,13 +12782,13 @@
         <v>837</v>
       </c>
       <c r="D45" s="5" t="s">
+        <v>901</v>
+      </c>
+      <c r="E45" s="5" t="s">
         <v>902</v>
       </c>
-      <c r="E45" s="5" t="s">
+      <c r="F45" s="5" t="s">
         <v>903</v>
-      </c>
-      <c r="F45" s="5" t="s">
-        <v>904</v>
       </c>
       <c r="G45" s="5"/>
       <c r="H45" s="5"/>
@@ -12780,7 +12797,7 @@
     </row>
     <row r="46" spans="1:10" ht="42" customHeight="1">
       <c r="A46" s="2" t="s">
-        <v>1040</v>
+        <v>1039</v>
       </c>
       <c r="B46" s="8">
         <v>2</v>
@@ -12795,7 +12812,7 @@
         <v>897</v>
       </c>
       <c r="F46" s="5" t="s">
-        <v>898</v>
+        <v>1189</v>
       </c>
       <c r="G46" s="5"/>
       <c r="H46" s="5"/>
@@ -12804,7 +12821,7 @@
     </row>
     <row r="47" spans="1:10" ht="42" customHeight="1">
       <c r="A47" s="2" t="s">
-        <v>1041</v>
+        <v>1040</v>
       </c>
       <c r="B47" s="8">
         <v>2</v>
@@ -12813,16 +12830,16 @@
         <v>837</v>
       </c>
       <c r="D47" s="5" t="s">
+        <v>958</v>
+      </c>
+      <c r="E47" s="5" t="s">
         <v>959</v>
       </c>
-      <c r="E47" s="5" t="s">
+      <c r="F47" s="5" t="s">
         <v>960</v>
       </c>
-      <c r="F47" s="5" t="s">
+      <c r="G47" s="5" t="s">
         <v>961</v>
-      </c>
-      <c r="G47" s="5" t="s">
-        <v>962</v>
       </c>
       <c r="H47" s="5"/>
       <c r="I47" s="5"/>
@@ -12830,7 +12847,7 @@
     </row>
     <row r="48" spans="1:10" ht="42" customHeight="1">
       <c r="A48" s="2" t="s">
-        <v>1042</v>
+        <v>1041</v>
       </c>
       <c r="B48" s="8">
         <v>2</v>
@@ -12852,7 +12869,7 @@
     </row>
     <row r="49" spans="1:10" ht="42" customHeight="1">
       <c r="A49" s="2" t="s">
-        <v>1043</v>
+        <v>1042</v>
       </c>
       <c r="B49" s="8">
         <v>2</v>
@@ -12861,13 +12878,13 @@
         <v>837</v>
       </c>
       <c r="D49" s="5" t="s">
-        <v>978</v>
+        <v>977</v>
       </c>
       <c r="E49" s="5" t="s">
+        <v>979</v>
+      </c>
+      <c r="F49" s="5" t="s">
         <v>980</v>
-      </c>
-      <c r="F49" s="5" t="s">
-        <v>981</v>
       </c>
       <c r="G49" s="5"/>
       <c r="H49" s="5"/>
@@ -12876,7 +12893,7 @@
     </row>
     <row r="50" spans="1:10" ht="42" customHeight="1">
       <c r="A50" s="2" t="s">
-        <v>1044</v>
+        <v>1043</v>
       </c>
       <c r="B50" s="8">
         <v>2</v>
@@ -12885,13 +12902,13 @@
         <v>837</v>
       </c>
       <c r="D50" s="5" t="s">
-        <v>979</v>
+        <v>978</v>
       </c>
       <c r="E50" s="5" t="s">
-        <v>983</v>
+        <v>982</v>
       </c>
       <c r="F50" s="5" t="s">
-        <v>982</v>
+        <v>981</v>
       </c>
       <c r="G50" s="5"/>
       <c r="H50" s="5"/>
@@ -12900,7 +12917,7 @@
     </row>
     <row r="51" spans="1:10" ht="42" customHeight="1">
       <c r="A51" s="2" t="s">
-        <v>1045</v>
+        <v>1044</v>
       </c>
       <c r="B51" s="8">
         <v>2</v>
@@ -12909,10 +12926,10 @@
         <v>837</v>
       </c>
       <c r="D51" s="5" t="s">
-        <v>972</v>
+        <v>971</v>
       </c>
       <c r="E51" s="5" t="s">
-        <v>974</v>
+        <v>973</v>
       </c>
       <c r="F51" s="5"/>
       <c r="G51" s="5"/>
@@ -12922,7 +12939,7 @@
     </row>
     <row r="52" spans="1:10" ht="42" customHeight="1">
       <c r="A52" s="2" t="s">
-        <v>1046</v>
+        <v>1045</v>
       </c>
       <c r="B52" s="8">
         <v>2</v>
@@ -12931,10 +12948,10 @@
         <v>837</v>
       </c>
       <c r="D52" s="5" t="s">
-        <v>971</v>
+        <v>970</v>
       </c>
       <c r="E52" s="5" t="s">
-        <v>973</v>
+        <v>972</v>
       </c>
       <c r="F52" s="5"/>
       <c r="G52" s="5"/>
@@ -12944,7 +12961,7 @@
     </row>
     <row r="53" spans="1:10" ht="42" customHeight="1">
       <c r="A53" s="2" t="s">
-        <v>1047</v>
+        <v>1046</v>
       </c>
       <c r="B53" s="8">
         <v>2</v>
@@ -12966,7 +12983,7 @@
     </row>
     <row r="54" spans="1:10" ht="42" customHeight="1">
       <c r="A54" s="2" t="s">
-        <v>1048</v>
+        <v>1047</v>
       </c>
       <c r="B54" s="7">
         <v>2</v>
@@ -12988,7 +13005,7 @@
     </row>
     <row r="55" spans="1:10" ht="42" customHeight="1">
       <c r="A55" s="2" t="s">
-        <v>1049</v>
+        <v>1048</v>
       </c>
       <c r="B55" s="8">
         <v>2</v>
@@ -13010,7 +13027,7 @@
     </row>
     <row r="56" spans="1:10" ht="42" customHeight="1">
       <c r="A56" s="2" t="s">
-        <v>1050</v>
+        <v>1049</v>
       </c>
       <c r="B56" s="8">
         <v>2</v>
@@ -13019,16 +13036,16 @@
         <v>837</v>
       </c>
       <c r="D56" s="5" t="s">
+        <v>930</v>
+      </c>
+      <c r="E56" s="5" t="s">
         <v>931</v>
       </c>
-      <c r="E56" s="5" t="s">
+      <c r="F56" s="5" t="s">
         <v>932</v>
       </c>
-      <c r="F56" s="5" t="s">
+      <c r="G56" s="5" t="s">
         <v>933</v>
-      </c>
-      <c r="G56" s="5" t="s">
-        <v>934</v>
       </c>
       <c r="H56" s="5"/>
       <c r="I56" s="5"/>
@@ -13036,7 +13053,7 @@
     </row>
     <row r="57" spans="1:10" ht="42" customHeight="1">
       <c r="A57" s="2" t="s">
-        <v>1051</v>
+        <v>1050</v>
       </c>
       <c r="B57" s="8">
         <v>2</v>
@@ -13060,7 +13077,7 @@
     </row>
     <row r="58" spans="1:10" ht="42" customHeight="1">
       <c r="A58" s="2" t="s">
-        <v>1052</v>
+        <v>1051</v>
       </c>
       <c r="B58" s="8">
         <v>2</v>
@@ -13069,13 +13086,13 @@
         <v>837</v>
       </c>
       <c r="D58" s="5" t="s">
+        <v>974</v>
+      </c>
+      <c r="E58" s="5" t="s">
+        <v>976</v>
+      </c>
+      <c r="F58" s="5" t="s">
         <v>975</v>
-      </c>
-      <c r="E58" s="5" t="s">
-        <v>977</v>
-      </c>
-      <c r="F58" s="5" t="s">
-        <v>976</v>
       </c>
       <c r="G58" s="5"/>
       <c r="H58" s="5"/>
@@ -13084,81 +13101,81 @@
     </row>
     <row r="59" spans="1:10" ht="42" customHeight="1">
       <c r="A59" s="2" t="s">
-        <v>1053</v>
+        <v>1052</v>
       </c>
       <c r="B59" s="7" t="s">
-        <v>995</v>
+        <v>994</v>
       </c>
       <c r="C59" s="7" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="D59" s="5" t="s">
-        <v>1114</v>
+        <v>1113</v>
       </c>
       <c r="E59" s="5" t="s">
+        <v>1108</v>
+      </c>
+      <c r="F59" s="5" t="s">
         <v>1109</v>
       </c>
-      <c r="F59" s="5" t="s">
+      <c r="G59" s="5" t="s">
         <v>1110</v>
       </c>
-      <c r="G59" s="5" t="s">
+      <c r="H59" s="5" t="s">
         <v>1111</v>
-      </c>
-      <c r="H59" s="5" t="s">
-        <v>1112</v>
       </c>
       <c r="I59" s="5"/>
       <c r="J59" s="5"/>
     </row>
     <row r="60" spans="1:10" ht="42" customHeight="1">
       <c r="A60" s="2" t="s">
-        <v>1054</v>
+        <v>1053</v>
       </c>
       <c r="B60" s="13" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="C60" s="7" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="D60" s="5" t="s">
-        <v>1113</v>
+        <v>1112</v>
       </c>
       <c r="E60" s="5" t="s">
+        <v>1115</v>
+      </c>
+      <c r="F60" s="5" t="s">
+        <v>1114</v>
+      </c>
+      <c r="G60" s="5" t="s">
         <v>1116</v>
       </c>
-      <c r="F60" s="5" t="s">
-        <v>1115</v>
-      </c>
-      <c r="G60" s="5" t="s">
+      <c r="H60" s="5" t="s">
         <v>1117</v>
-      </c>
-      <c r="H60" s="5" t="s">
-        <v>1118</v>
       </c>
       <c r="I60" s="5"/>
       <c r="J60" s="5"/>
     </row>
     <row r="61" spans="1:10" ht="42" customHeight="1">
       <c r="A61" s="2" t="s">
-        <v>1055</v>
+        <v>1054</v>
       </c>
       <c r="B61" s="13" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="C61" s="7" t="s">
-        <v>1068</v>
+        <v>1067</v>
       </c>
       <c r="D61" s="5" t="s">
+        <v>1118</v>
+      </c>
+      <c r="E61" s="5" t="s">
         <v>1119</v>
       </c>
-      <c r="E61" s="5" t="s">
+      <c r="F61" s="5" t="s">
         <v>1120</v>
       </c>
-      <c r="F61" s="5" t="s">
+      <c r="G61" s="5" t="s">
         <v>1121</v>
-      </c>
-      <c r="G61" s="5" t="s">
-        <v>1122</v>
       </c>
       <c r="H61" s="5"/>
       <c r="I61" s="5"/>
@@ -13166,25 +13183,25 @@
     </row>
     <row r="62" spans="1:10" ht="42" customHeight="1">
       <c r="A62" s="2" t="s">
-        <v>1056</v>
+        <v>1055</v>
       </c>
       <c r="B62" s="13" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="C62" s="7" t="s">
+        <v>1125</v>
+      </c>
+      <c r="D62" s="5" t="s">
         <v>1126</v>
       </c>
-      <c r="D62" s="5" t="s">
+      <c r="E62" s="5" t="s">
         <v>1127</v>
       </c>
-      <c r="E62" s="5" t="s">
+      <c r="F62" s="5" t="s">
         <v>1128</v>
       </c>
-      <c r="F62" s="5" t="s">
+      <c r="G62" s="5" t="s">
         <v>1129</v>
-      </c>
-      <c r="G62" s="5" t="s">
-        <v>1130</v>
       </c>
       <c r="H62" s="5"/>
       <c r="I62" s="5"/>
@@ -13192,13 +13209,13 @@
     </row>
     <row r="63" spans="1:10" ht="42" customHeight="1">
       <c r="A63" s="2" t="s">
-        <v>1057</v>
+        <v>1056</v>
       </c>
       <c r="B63" s="13" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="C63" s="7" t="s">
-        <v>1126</v>
+        <v>1125</v>
       </c>
       <c r="D63" s="5" t="s">
         <v>561</v>
@@ -13214,13 +13231,13 @@
     </row>
     <row r="64" spans="1:10" ht="42" customHeight="1">
       <c r="A64" s="2" t="s">
-        <v>1058</v>
+        <v>1057</v>
       </c>
       <c r="B64" s="13" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="C64" s="7" t="s">
-        <v>1126</v>
+        <v>1125</v>
       </c>
       <c r="D64" s="5" t="s">
         <v>564</v>
@@ -13236,13 +13253,13 @@
     </row>
     <row r="65" spans="1:10" ht="42" customHeight="1">
       <c r="A65" s="2" t="s">
-        <v>1059</v>
+        <v>1058</v>
       </c>
       <c r="B65" s="13" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="C65" s="7" t="s">
-        <v>1126</v>
+        <v>1125</v>
       </c>
       <c r="D65" s="5" t="s">
         <v>567</v>
@@ -13260,49 +13277,49 @@
     </row>
     <row r="66" spans="1:10" ht="42" customHeight="1">
       <c r="A66" s="2" t="s">
-        <v>1060</v>
+        <v>1059</v>
       </c>
       <c r="B66" s="7" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="C66" s="7" t="s">
-        <v>1124</v>
+        <v>1123</v>
       </c>
       <c r="D66" s="5" t="s">
+        <v>1068</v>
+      </c>
+      <c r="E66" s="5" t="s">
         <v>1069</v>
       </c>
-      <c r="E66" s="5" t="s">
+      <c r="F66" s="5" t="s">
+        <v>1187</v>
+      </c>
+      <c r="G66" s="5" t="s">
         <v>1070</v>
       </c>
-      <c r="F66" s="5" t="s">
-        <v>1188</v>
-      </c>
-      <c r="G66" s="5" t="s">
+      <c r="H66" s="5" t="s">
         <v>1071</v>
       </c>
-      <c r="H66" s="5" t="s">
+      <c r="I66" s="5" t="s">
         <v>1072</v>
-      </c>
-      <c r="I66" s="5" t="s">
-        <v>1073</v>
       </c>
       <c r="J66" s="5"/>
     </row>
     <row r="67" spans="1:10" ht="42" customHeight="1">
       <c r="A67" s="2" t="s">
-        <v>1061</v>
+        <v>1060</v>
       </c>
       <c r="B67" s="13" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="C67" s="7" t="s">
-        <v>1124</v>
+        <v>1123</v>
       </c>
       <c r="D67" s="5" t="s">
+        <v>1073</v>
+      </c>
+      <c r="E67" s="5" t="s">
         <v>1074</v>
-      </c>
-      <c r="E67" s="5" t="s">
-        <v>1075</v>
       </c>
       <c r="F67" s="5"/>
       <c r="G67" s="5"/>
@@ -13312,22 +13329,22 @@
     </row>
     <row r="68" spans="1:10" ht="42" customHeight="1">
       <c r="A68" s="2" t="s">
-        <v>1062</v>
+        <v>1061</v>
       </c>
       <c r="B68" s="13" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="C68" s="7" t="s">
-        <v>1124</v>
+        <v>1123</v>
       </c>
       <c r="D68" s="5" t="s">
+        <v>1075</v>
+      </c>
+      <c r="E68" s="5" t="s">
         <v>1076</v>
       </c>
-      <c r="E68" s="5" t="s">
-        <v>1077</v>
-      </c>
       <c r="F68" s="5" t="s">
-        <v>1189</v>
+        <v>1188</v>
       </c>
       <c r="G68" s="5"/>
       <c r="H68" s="5"/>
@@ -13336,19 +13353,19 @@
     </row>
     <row r="69" spans="1:10" ht="42" customHeight="1">
       <c r="A69" s="2" t="s">
-        <v>1063</v>
+        <v>1062</v>
       </c>
       <c r="B69" s="13" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="C69" s="7" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
       <c r="D69" s="5" t="s">
-        <v>1078</v>
+        <v>1077</v>
       </c>
       <c r="E69" s="5" t="s">
-        <v>1080</v>
+        <v>1079</v>
       </c>
       <c r="F69" s="5"/>
       <c r="G69" s="5"/>
@@ -13358,19 +13375,19 @@
     </row>
     <row r="70" spans="1:10" ht="42" customHeight="1">
       <c r="A70" s="2" t="s">
-        <v>1064</v>
+        <v>1063</v>
       </c>
       <c r="B70" s="13" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="C70" s="7" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
       <c r="D70" s="5" t="s">
-        <v>1079</v>
+        <v>1078</v>
       </c>
       <c r="E70" s="5" t="s">
-        <v>1081</v>
+        <v>1080</v>
       </c>
       <c r="F70" s="5"/>
       <c r="G70" s="5"/>
@@ -13380,19 +13397,19 @@
     </row>
     <row r="71" spans="1:10" ht="42" customHeight="1">
       <c r="A71" s="2" t="s">
-        <v>1065</v>
+        <v>1064</v>
       </c>
       <c r="B71" s="13" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="C71" s="7" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
       <c r="D71" s="5" t="s">
+        <v>1081</v>
+      </c>
+      <c r="E71" s="5" t="s">
         <v>1082</v>
-      </c>
-      <c r="E71" s="5" t="s">
-        <v>1083</v>
       </c>
       <c r="F71" s="5"/>
       <c r="G71" s="5"/>
@@ -13402,50 +13419,50 @@
     </row>
     <row r="72" spans="1:10" ht="42" customHeight="1">
       <c r="A72" s="2" t="s">
-        <v>1066</v>
+        <v>1065</v>
       </c>
       <c r="B72" s="13" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="C72" s="7" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
       <c r="D72" s="5" t="s">
+        <v>1083</v>
+      </c>
+      <c r="E72" s="5" t="s">
         <v>1084</v>
       </c>
-      <c r="E72" s="5" t="s">
+      <c r="F72" s="5" t="s">
         <v>1085</v>
       </c>
-      <c r="F72" s="5" t="s">
+      <c r="G72" s="5" t="s">
         <v>1086</v>
       </c>
-      <c r="G72" s="5" t="s">
+      <c r="H72" s="5" t="s">
         <v>1087</v>
-      </c>
-      <c r="H72" s="5" t="s">
-        <v>1088</v>
       </c>
       <c r="I72" s="5"/>
       <c r="J72" s="5"/>
     </row>
     <row r="73" spans="1:10" ht="42" customHeight="1">
       <c r="A73" s="2" t="s">
-        <v>1067</v>
+        <v>1066</v>
       </c>
       <c r="B73" s="13" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="C73" s="7" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
       <c r="D73" s="5" t="s">
-        <v>1091</v>
+        <v>1090</v>
       </c>
       <c r="E73" s="5" t="s">
+        <v>1088</v>
+      </c>
+      <c r="F73" s="5" t="s">
         <v>1089</v>
-      </c>
-      <c r="F73" s="5" t="s">
-        <v>1090</v>
       </c>
       <c r="G73" s="5"/>
       <c r="H73" s="5"/>
@@ -13454,22 +13471,22 @@
     </row>
     <row r="74" spans="1:10" ht="42" customHeight="1">
       <c r="A74" s="2" t="s">
-        <v>1171</v>
+        <v>1170</v>
       </c>
       <c r="B74" s="13" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="C74" s="7" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
       <c r="D74" s="5" t="s">
+        <v>1091</v>
+      </c>
+      <c r="E74" s="5" t="s">
         <v>1092</v>
       </c>
-      <c r="E74" s="5" t="s">
+      <c r="F74" s="5" t="s">
         <v>1093</v>
-      </c>
-      <c r="F74" s="5" t="s">
-        <v>1094</v>
       </c>
       <c r="G74" s="5"/>
       <c r="H74" s="5"/>
@@ -13478,22 +13495,22 @@
     </row>
     <row r="75" spans="1:10" ht="42" customHeight="1">
       <c r="A75" s="2" t="s">
-        <v>1172</v>
+        <v>1171</v>
       </c>
       <c r="B75" s="13" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="C75" s="7" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
       <c r="D75" s="5" t="s">
-        <v>1095</v>
+        <v>1094</v>
       </c>
       <c r="E75" s="5" t="s">
+        <v>1096</v>
+      </c>
+      <c r="F75" s="5" t="s">
         <v>1097</v>
-      </c>
-      <c r="F75" s="5" t="s">
-        <v>1098</v>
       </c>
       <c r="G75" s="5"/>
       <c r="H75" s="5"/>
@@ -13502,19 +13519,19 @@
     </row>
     <row r="76" spans="1:10" ht="42" customHeight="1">
       <c r="A76" s="2" t="s">
-        <v>1173</v>
+        <v>1172</v>
       </c>
       <c r="B76" s="13" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="C76" s="7" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
       <c r="D76" s="5" t="s">
-        <v>1096</v>
+        <v>1095</v>
       </c>
       <c r="E76" s="5" t="s">
-        <v>1099</v>
+        <v>1098</v>
       </c>
       <c r="F76" s="5"/>
       <c r="G76" s="5"/>
@@ -13524,53 +13541,53 @@
     </row>
     <row r="77" spans="1:10" ht="42" customHeight="1">
       <c r="A77" s="2" t="s">
-        <v>1174</v>
+        <v>1173</v>
       </c>
       <c r="B77" s="13" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="C77" s="7" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
       <c r="D77" s="5" t="s">
+        <v>1099</v>
+      </c>
+      <c r="E77" s="5" t="s">
         <v>1100</v>
       </c>
-      <c r="E77" s="5" t="s">
+      <c r="F77" s="5" t="s">
         <v>1101</v>
       </c>
-      <c r="F77" s="5" t="s">
+      <c r="G77" s="5" t="s">
         <v>1102</v>
       </c>
-      <c r="G77" s="5" t="s">
+      <c r="H77" s="5" t="s">
         <v>1103</v>
-      </c>
-      <c r="H77" s="5" t="s">
-        <v>1104</v>
       </c>
       <c r="I77" s="5"/>
       <c r="J77" s="5"/>
     </row>
     <row r="78" spans="1:10" ht="42" customHeight="1">
       <c r="A78" s="2" t="s">
-        <v>1175</v>
+        <v>1174</v>
       </c>
       <c r="B78" s="13" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="C78" s="7" t="s">
-        <v>1123</v>
+        <v>1122</v>
       </c>
       <c r="D78" s="5" t="s">
+        <v>1104</v>
+      </c>
+      <c r="E78" s="5" t="s">
         <v>1105</v>
       </c>
-      <c r="E78" s="5" t="s">
+      <c r="F78" s="5" t="s">
         <v>1106</v>
       </c>
-      <c r="F78" s="5" t="s">
+      <c r="G78" s="5" t="s">
         <v>1107</v>
-      </c>
-      <c r="G78" s="5" t="s">
-        <v>1108</v>
       </c>
       <c r="H78" s="5"/>
       <c r="I78" s="5"/>
@@ -13578,22 +13595,22 @@
     </row>
     <row r="79" spans="1:10" ht="42" customHeight="1">
       <c r="A79" s="2" t="s">
-        <v>1176</v>
+        <v>1175</v>
       </c>
       <c r="B79" s="7" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="C79" s="7" t="s">
-        <v>1125</v>
+        <v>1124</v>
       </c>
       <c r="D79" s="5" t="s">
+        <v>1130</v>
+      </c>
+      <c r="E79" s="5" t="s">
         <v>1131</v>
       </c>
-      <c r="E79" s="5" t="s">
+      <c r="F79" s="5" t="s">
         <v>1132</v>
-      </c>
-      <c r="F79" s="5" t="s">
-        <v>1133</v>
       </c>
       <c r="G79" s="5"/>
       <c r="H79" s="5"/>
@@ -13602,22 +13619,22 @@
     </row>
     <row r="80" spans="1:10" ht="42" customHeight="1">
       <c r="A80" s="2" t="s">
-        <v>1177</v>
+        <v>1176</v>
       </c>
       <c r="B80" s="13" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="C80" s="7" t="s">
-        <v>1125</v>
+        <v>1124</v>
       </c>
       <c r="D80" s="5" t="s">
+        <v>1133</v>
+      </c>
+      <c r="E80" s="5" t="s">
         <v>1134</v>
       </c>
-      <c r="E80" s="5" t="s">
+      <c r="F80" s="5" t="s">
         <v>1135</v>
-      </c>
-      <c r="F80" s="5" t="s">
-        <v>1136</v>
       </c>
       <c r="G80" s="5"/>
       <c r="H80" s="5"/>
@@ -13626,25 +13643,25 @@
     </row>
     <row r="81" spans="1:10" ht="42" customHeight="1">
       <c r="A81" s="2" t="s">
-        <v>1178</v>
+        <v>1177</v>
       </c>
       <c r="B81" s="7" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="C81" s="7" t="s">
-        <v>1125</v>
+        <v>1124</v>
       </c>
       <c r="D81" s="5" t="s">
+        <v>1136</v>
+      </c>
+      <c r="E81" s="5" t="s">
         <v>1137</v>
       </c>
-      <c r="E81" s="5" t="s">
+      <c r="F81" s="5" t="s">
         <v>1138</v>
       </c>
-      <c r="F81" s="5" t="s">
+      <c r="G81" s="5" t="s">
         <v>1139</v>
-      </c>
-      <c r="G81" s="5" t="s">
-        <v>1140</v>
       </c>
       <c r="H81" s="5"/>
       <c r="I81" s="5"/>
@@ -13652,22 +13669,22 @@
     </row>
     <row r="82" spans="1:10" ht="42" customHeight="1">
       <c r="A82" s="2" t="s">
-        <v>1179</v>
+        <v>1178</v>
       </c>
       <c r="B82" s="13" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="C82" s="7" t="s">
-        <v>1125</v>
+        <v>1124</v>
       </c>
       <c r="D82" s="5" t="s">
-        <v>1143</v>
+        <v>1142</v>
       </c>
       <c r="E82" s="5" t="s">
+        <v>1140</v>
+      </c>
+      <c r="F82" s="5" t="s">
         <v>1141</v>
-      </c>
-      <c r="F82" s="5" t="s">
-        <v>1142</v>
       </c>
       <c r="G82" s="5"/>
       <c r="H82" s="5"/>
@@ -13676,19 +13693,19 @@
     </row>
     <row r="83" spans="1:10" ht="42" customHeight="1">
       <c r="A83" s="2" t="s">
-        <v>1180</v>
+        <v>1179</v>
       </c>
       <c r="B83" s="7" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="C83" s="7" t="s">
-        <v>1125</v>
+        <v>1124</v>
       </c>
       <c r="D83" s="5" t="s">
+        <v>1143</v>
+      </c>
+      <c r="E83" s="5" t="s">
         <v>1144</v>
-      </c>
-      <c r="E83" s="5" t="s">
-        <v>1145</v>
       </c>
       <c r="F83" s="5"/>
       <c r="G83" s="5"/>
@@ -13698,25 +13715,25 @@
     </row>
     <row r="84" spans="1:10" ht="42" customHeight="1">
       <c r="A84" s="2" t="s">
-        <v>1181</v>
+        <v>1180</v>
       </c>
       <c r="B84" s="13" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="C84" s="7" t="s">
-        <v>1125</v>
+        <v>1124</v>
       </c>
       <c r="D84" s="5" t="s">
+        <v>1145</v>
+      </c>
+      <c r="E84" s="5" t="s">
         <v>1146</v>
       </c>
-      <c r="E84" s="5" t="s">
+      <c r="F84" s="5" t="s">
         <v>1147</v>
       </c>
-      <c r="F84" s="5" t="s">
+      <c r="G84" s="5" t="s">
         <v>1148</v>
-      </c>
-      <c r="G84" s="5" t="s">
-        <v>1149</v>
       </c>
       <c r="H84" s="5"/>
       <c r="I84" s="5"/>
@@ -13724,22 +13741,22 @@
     </row>
     <row r="85" spans="1:10" ht="42" customHeight="1">
       <c r="A85" s="2" t="s">
-        <v>1182</v>
+        <v>1181</v>
       </c>
       <c r="B85" s="7" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="C85" s="7" t="s">
-        <v>1125</v>
+        <v>1124</v>
       </c>
       <c r="D85" s="5" t="s">
+        <v>1149</v>
+      </c>
+      <c r="E85" s="5" t="s">
         <v>1150</v>
       </c>
-      <c r="E85" s="5" t="s">
+      <c r="F85" s="5" t="s">
         <v>1151</v>
-      </c>
-      <c r="F85" s="5" t="s">
-        <v>1152</v>
       </c>
       <c r="G85" s="5"/>
       <c r="H85" s="5"/>
@@ -13748,108 +13765,108 @@
     </row>
     <row r="86" spans="1:10" ht="42" customHeight="1">
       <c r="A86" s="2" t="s">
-        <v>1183</v>
+        <v>1182</v>
       </c>
       <c r="B86" s="13" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="C86" s="7" t="s">
-        <v>1125</v>
+        <v>1124</v>
       </c>
       <c r="D86" s="5" t="s">
+        <v>1152</v>
+      </c>
+      <c r="E86" s="5" t="s">
         <v>1153</v>
       </c>
-      <c r="E86" s="5" t="s">
+      <c r="F86" s="5" t="s">
         <v>1154</v>
       </c>
-      <c r="F86" s="5" t="s">
+      <c r="G86" s="5" t="s">
         <v>1155</v>
       </c>
-      <c r="G86" s="5" t="s">
+      <c r="H86" s="5" t="s">
         <v>1156</v>
-      </c>
-      <c r="H86" s="5" t="s">
-        <v>1157</v>
       </c>
       <c r="I86" s="5"/>
       <c r="J86" s="5"/>
     </row>
     <row r="87" spans="1:10" ht="42" customHeight="1">
       <c r="A87" s="2" t="s">
-        <v>1184</v>
+        <v>1183</v>
       </c>
       <c r="B87" s="7" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="C87" s="7" t="s">
-        <v>1125</v>
+        <v>1124</v>
       </c>
       <c r="D87" s="5" t="s">
+        <v>1157</v>
+      </c>
+      <c r="E87" s="5" t="s">
         <v>1158</v>
       </c>
-      <c r="E87" s="5" t="s">
+      <c r="F87" s="5" t="s">
         <v>1159</v>
       </c>
-      <c r="F87" s="5" t="s">
+      <c r="G87" s="5" t="s">
         <v>1160</v>
       </c>
-      <c r="G87" s="5" t="s">
-        <v>1161</v>
-      </c>
       <c r="H87" s="5" t="s">
-        <v>1157</v>
+        <v>1156</v>
       </c>
       <c r="I87" s="5"/>
       <c r="J87" s="5"/>
     </row>
     <row r="88" spans="1:10" ht="42" customHeight="1">
       <c r="A88" s="2" t="s">
-        <v>1185</v>
+        <v>1184</v>
       </c>
       <c r="B88" s="13" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="C88" s="7" t="s">
-        <v>1125</v>
+        <v>1124</v>
       </c>
       <c r="D88" s="5" t="s">
+        <v>1161</v>
+      </c>
+      <c r="E88" s="5" t="s">
         <v>1162</v>
       </c>
-      <c r="E88" s="5" t="s">
+      <c r="F88" s="5" t="s">
         <v>1163</v>
       </c>
-      <c r="F88" s="5" t="s">
+      <c r="G88" s="5" t="s">
         <v>1164</v>
       </c>
-      <c r="G88" s="5" t="s">
+      <c r="H88" s="5" t="s">
         <v>1165</v>
       </c>
-      <c r="H88" s="5" t="s">
+      <c r="I88" s="5" t="s">
         <v>1166</v>
-      </c>
-      <c r="I88" s="5" t="s">
-        <v>1167</v>
       </c>
       <c r="J88" s="5"/>
     </row>
     <row r="89" spans="1:10" ht="42" customHeight="1">
       <c r="A89" s="2" t="s">
-        <v>1186</v>
+        <v>1185</v>
       </c>
       <c r="B89" s="7" t="s">
-        <v>994</v>
+        <v>993</v>
       </c>
       <c r="C89" s="7" t="s">
-        <v>1125</v>
+        <v>1124</v>
       </c>
       <c r="D89" s="5" t="s">
+        <v>1167</v>
+      </c>
+      <c r="E89" s="5" t="s">
         <v>1168</v>
       </c>
-      <c r="E89" s="5" t="s">
+      <c r="F89" s="5" t="s">
         <v>1169</v>
-      </c>
-      <c r="F89" s="5" t="s">
-        <v>1170</v>
       </c>
       <c r="G89" s="5"/>
       <c r="H89" s="5"/>

</xml_diff>